<commit_message>
Add Trackslot-Xorwow processed results
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AC914C-E66D-1048-BC6D-87AF01B02D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6763BE09-8245-9046-A2DC-9ED198AEE670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38980" yWindow="1380" windowWidth="40000" windowHeight="21680" activeTab="1" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
+    <workbookView xWindow="38980" yWindow="1380" windowWidth="40000" windowHeight="21680" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_Results" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="22">
   <si>
     <t>Branch</t>
   </si>
@@ -103,13 +103,16 @@
   </si>
   <si>
     <t>Run</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -119,6 +122,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -145,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -156,6 +165,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B71848BA-D8C3-7041-A0EE-B663A4811CD2}">
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="42.1640625" bestFit="1" customWidth="1"/>
@@ -674,6 +684,48 @@
       <c r="B4" t="s">
         <v>3</v>
       </c>
+      <c r="C4" s="6">
+        <v>4.7361520297999897</v>
+      </c>
+      <c r="E4" s="6">
+        <v>21.1806411148</v>
+      </c>
+      <c r="G4" s="6">
+        <v>9.4521483475999908</v>
+      </c>
+      <c r="I4" s="6">
+        <v>6.2249833689000003</v>
+      </c>
+      <c r="K4" s="6">
+        <v>4.7699677447999997</v>
+      </c>
+      <c r="M4" s="6">
+        <v>4.7879055426999999</v>
+      </c>
+      <c r="O4" s="6">
+        <v>4.8561072632000002</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>4.9457645918999997</v>
+      </c>
+      <c r="S4" s="6">
+        <v>4.8490968258999896</v>
+      </c>
+      <c r="U4" s="6">
+        <v>10.3908139883</v>
+      </c>
+      <c r="W4" s="6">
+        <v>4.7319136024999997</v>
+      </c>
+      <c r="Y4" s="6">
+        <v>0.56397134309999997</v>
+      </c>
+      <c r="AA4" s="6">
+        <v>80.952135558099997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="N14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -698,7 +750,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D90E2C0-8C68-E84F-BBAA-6A32D2F1D90D}">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="42.1640625" bestFit="1" customWidth="1"/>
@@ -722,21 +774,6 @@
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -754,102 +791,553 @@
       <c r="AB2" s="2"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>4.7340293059999903</v>
+      </c>
+      <c r="D5">
+        <v>21.176729871999999</v>
+      </c>
+      <c r="E5">
+        <v>9.4457361899999892</v>
+      </c>
+      <c r="F5">
+        <v>6.2217804140000004</v>
+      </c>
+      <c r="G5">
+        <v>4.7682641119999998</v>
+      </c>
+      <c r="H5">
+        <v>4.78634752199999</v>
+      </c>
+      <c r="I5">
+        <v>4.8526370550000104</v>
+      </c>
+      <c r="J5">
+        <v>4.9441060699999904</v>
+      </c>
+      <c r="K5">
+        <v>4.8479211129999804</v>
+      </c>
+      <c r="L5">
+        <v>10.389432319999999</v>
+      </c>
+      <c r="M5">
+        <v>4.73018520599999</v>
+      </c>
+      <c r="N5">
+        <v>0.57304119499999995</v>
+      </c>
+      <c r="O5">
+        <v>80.923910221</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>4.7393095049999996</v>
+      </c>
+      <c r="D6">
+        <v>21.173363765999898</v>
+      </c>
+      <c r="E6">
+        <v>9.4572644579999796</v>
+      </c>
+      <c r="F6">
+        <v>6.2261814449999999</v>
+      </c>
+      <c r="G6">
+        <v>4.7731040329999903</v>
+      </c>
+      <c r="H6">
+        <v>4.7896122209999898</v>
+      </c>
+      <c r="I6">
+        <v>4.8602087559999996</v>
+      </c>
+      <c r="J6">
+        <v>4.9492782460000004</v>
+      </c>
+      <c r="K6">
+        <v>4.8529851260000001</v>
+      </c>
+      <c r="L6">
+        <v>10.393453508</v>
+      </c>
+      <c r="M6">
+        <v>4.7350227470000004</v>
+      </c>
+      <c r="N6">
+        <v>0.57079999699999995</v>
+      </c>
+      <c r="O6">
+        <v>80.976149698</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B7">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>4.7078935550000001</v>
+      </c>
+      <c r="D7">
+        <v>21.146499433999999</v>
+      </c>
+      <c r="E7">
+        <v>9.3944941359999898</v>
+      </c>
+      <c r="F7">
+        <v>6.1949537149999996</v>
+      </c>
+      <c r="G7">
+        <v>4.7398854799999999</v>
+      </c>
+      <c r="H7">
+        <v>4.7574510490000002</v>
+      </c>
+      <c r="I7">
+        <v>4.8284425640000102</v>
+      </c>
+      <c r="J7">
+        <v>4.9171688830000102</v>
+      </c>
+      <c r="K7">
+        <v>4.8211042189999898</v>
+      </c>
+      <c r="L7">
+        <v>10.363234916</v>
+      </c>
+      <c r="M7">
+        <v>4.7036561429999999</v>
+      </c>
+      <c r="N7">
+        <v>0.57259144100000003</v>
+      </c>
+      <c r="O7">
+        <v>80.601453527000004</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B8">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>4.8357023659999996</v>
+      </c>
+      <c r="D8">
+        <v>21.283297358999999</v>
+      </c>
+      <c r="E8">
+        <v>9.6534851180000008</v>
+      </c>
+      <c r="F8">
+        <v>6.3259116600000098</v>
+      </c>
+      <c r="G8">
+        <v>4.8699703429999897</v>
+      </c>
+      <c r="H8">
+        <v>4.8880030239999899</v>
+      </c>
+      <c r="I8">
+        <v>4.9540698719999998</v>
+      </c>
+      <c r="J8">
+        <v>5.0477363430000004</v>
+      </c>
+      <c r="K8">
+        <v>4.9493739049999999</v>
+      </c>
+      <c r="L8">
+        <v>10.490154618999901</v>
+      </c>
+      <c r="M8">
+        <v>4.8317443500000001</v>
+      </c>
+      <c r="N8">
+        <v>0.56438216600000002</v>
+      </c>
+      <c r="O8">
+        <v>82.156601383999998</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B9">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>4.7201029639999899</v>
+      </c>
+      <c r="D9">
+        <v>21.162477132999999</v>
+      </c>
+      <c r="E9">
+        <v>9.4234756789999992</v>
+      </c>
+      <c r="F9">
+        <v>6.2093324299999804</v>
+      </c>
+      <c r="G9">
+        <v>4.7542486399999904</v>
+      </c>
+      <c r="H9">
+        <v>4.7723286930000004</v>
+      </c>
+      <c r="I9">
+        <v>4.8406304889999996</v>
+      </c>
+      <c r="J9">
+        <v>4.92910223999999</v>
+      </c>
+      <c r="K9">
+        <v>4.8331939989999997</v>
+      </c>
+      <c r="L9">
+        <v>10.376906498999899</v>
+      </c>
+      <c r="M9">
+        <v>4.7158174270000002</v>
+      </c>
+      <c r="N9">
+        <v>0.57460502199999997</v>
+      </c>
+      <c r="O9">
+        <v>80.764317835</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B10">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>4.7483563999999898</v>
+      </c>
+      <c r="D10">
+        <v>21.204867498999899</v>
+      </c>
+      <c r="E10">
+        <v>9.4793780250000097</v>
+      </c>
+      <c r="F10">
+        <v>6.2381119399999996</v>
+      </c>
+      <c r="G10">
+        <v>4.7830271779999904</v>
+      </c>
+      <c r="H10">
+        <v>4.8021576899999898</v>
+      </c>
+      <c r="I10">
+        <v>4.8694124350000001</v>
+      </c>
+      <c r="J10">
+        <v>4.9590571159999897</v>
+      </c>
+      <c r="K10">
+        <v>4.8623519149999801</v>
+      </c>
+      <c r="L10">
+        <v>10.401261198</v>
+      </c>
+      <c r="M10">
+        <v>4.74394939799999</v>
+      </c>
+      <c r="N10">
+        <v>0.55289784900000005</v>
+      </c>
+      <c r="O10">
+        <v>81.118364749999998</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B11">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>4.7037826629999904</v>
+      </c>
+      <c r="D11">
+        <v>21.152131596</v>
+      </c>
+      <c r="E11">
+        <v>9.3876109779999997</v>
+      </c>
+      <c r="F11">
+        <v>6.1921738199999998</v>
+      </c>
+      <c r="G11">
+        <v>4.73704256899999</v>
+      </c>
+      <c r="H11">
+        <v>4.7546049190000099</v>
+      </c>
+      <c r="I11">
+        <v>4.8231421749999903</v>
+      </c>
+      <c r="J11">
+        <v>4.9121940719999904</v>
+      </c>
+      <c r="K11">
+        <v>4.8161531389999999</v>
+      </c>
+      <c r="L11">
+        <v>10.356330882</v>
+      </c>
+      <c r="M11">
+        <v>4.6991199909999901</v>
+      </c>
+      <c r="N11">
+        <v>0.55554261299999996</v>
+      </c>
+      <c r="O11">
+        <v>80.560378224999994</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B12">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>4.6960157959999904</v>
+      </c>
+      <c r="D12">
+        <v>21.135143617000001</v>
+      </c>
+      <c r="E12">
+        <v>9.3704731389999907</v>
+      </c>
+      <c r="F12">
+        <v>6.1849777839999902</v>
+      </c>
+      <c r="G12">
+        <v>4.7298488310000097</v>
+      </c>
+      <c r="H12">
+        <v>4.74821225899999</v>
+      </c>
+      <c r="I12">
+        <v>4.8161023499999898</v>
+      </c>
+      <c r="J12">
+        <v>4.9041083179999996</v>
+      </c>
+      <c r="K12">
+        <v>4.8065764169999996</v>
+      </c>
+      <c r="L12">
+        <v>10.353393854</v>
+      </c>
+      <c r="M12">
+        <v>4.6916778209999901</v>
+      </c>
+      <c r="N12">
+        <v>0.55554574300000004</v>
+      </c>
+      <c r="O12">
+        <v>80.462678502000003</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>4.7152222879999997</v>
+      </c>
+      <c r="D13">
+        <v>21.163150134999899</v>
+      </c>
+      <c r="E13">
+        <v>9.4112512409999898</v>
+      </c>
+      <c r="F13">
+        <v>6.2047871109999999</v>
+      </c>
+      <c r="G13">
+        <v>4.7493141909999999</v>
+      </c>
+      <c r="H13">
+        <v>4.7671523330000003</v>
+      </c>
+      <c r="I13">
+        <v>4.8345936519999997</v>
+      </c>
+      <c r="J13">
+        <v>4.9243923099999902</v>
+      </c>
+      <c r="K13">
+        <v>4.8269851900000003</v>
+      </c>
+      <c r="L13">
+        <v>10.369362314</v>
+      </c>
+      <c r="M13">
+        <v>4.7109683779999898</v>
+      </c>
+      <c r="N13">
+        <v>0.56577272000000001</v>
+      </c>
+      <c r="O13">
+        <v>80.705057595</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B14">
         <v>9</v>
+      </c>
+      <c r="C14">
+        <v>4.7611054549999903</v>
+      </c>
+      <c r="D14">
+        <v>21.208750736999999</v>
+      </c>
+      <c r="E14">
+        <v>9.4983145119999808</v>
+      </c>
+      <c r="F14">
+        <v>6.2516233699999999</v>
+      </c>
+      <c r="G14">
+        <v>4.7949720709999903</v>
+      </c>
+      <c r="H14">
+        <v>4.8131857169999996</v>
+      </c>
+      <c r="I14">
+        <v>4.8818332839999803</v>
+      </c>
+      <c r="J14">
+        <v>4.9705023209999997</v>
+      </c>
+      <c r="K14">
+        <v>4.8743232359999897</v>
+      </c>
+      <c r="L14">
+        <v>10.414609773</v>
+      </c>
+      <c r="M14">
+        <v>4.7569945640000002</v>
+      </c>
+      <c r="N14">
+        <v>0.55453468500000003</v>
+      </c>
+      <c r="O14">
+        <v>81.252443843999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="B15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="3">
+        <v>4.7361520297999897</v>
+      </c>
+      <c r="D15" s="3">
+        <v>21.1806411148</v>
+      </c>
+      <c r="E15" s="3">
+        <v>9.4521483475999908</v>
+      </c>
+      <c r="F15" s="3">
+        <v>6.2249833689000003</v>
+      </c>
+      <c r="G15" s="3">
+        <v>4.7699677447999997</v>
+      </c>
+      <c r="H15" s="3">
+        <v>4.7879055426999999</v>
+      </c>
+      <c r="I15" s="3">
+        <v>4.8561072632000002</v>
+      </c>
+      <c r="J15" s="3">
+        <v>4.9457645918999997</v>
+      </c>
+      <c r="K15" s="3">
+        <v>4.8490968258999896</v>
+      </c>
+      <c r="L15" s="3">
+        <v>10.3908139883</v>
+      </c>
+      <c r="M15" s="3">
+        <v>4.7319136024999997</v>
+      </c>
+      <c r="N15" s="3">
+        <v>0.56397134309999997</v>
+      </c>
+      <c r="O15" s="3">
+        <v>80.952135558099997</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C1:O1"/>
+    <mergeCell ref="C3:O3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add timings from track-xorwow and analysis worksheet
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F6BD87-1522-1041-BDA5-C1C1F92C82C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA1CDE0-9160-0642-80B2-BA4607FE6B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38240" yWindow="1520" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
+    <workbookView xWindow="43100" yWindow="1360" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_Results" sheetId="1" r:id="rId1"/>
     <sheet name="Trackslot_Xorwow" sheetId="2" r:id="rId2"/>
     <sheet name="Trackslot_Ranluxpp" sheetId="3" r:id="rId3"/>
+    <sheet name="Track_Xorwow" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="26">
   <si>
     <t>Branch</t>
   </si>
@@ -113,6 +114,12 @@
   </si>
   <si>
     <t>Rel Diff (%)</t>
+  </si>
+  <si>
+    <t>Trackslot reseeding</t>
+  </si>
+  <si>
+    <t>Track reseeding</t>
   </si>
 </sst>
 </file>
@@ -521,6 +528,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
@@ -564,11 +577,11 @@
       <c r="AO1" s="4"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>5</v>
@@ -756,11 +769,8 @@
       </c>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2">
         <v>4.7361520297999897</v>
@@ -893,7 +903,54 @@
         <v>74.415986674081395</v>
       </c>
     </row>
+    <row r="5" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2.0490970599999998E-2</v>
+      </c>
+      <c r="F5" s="1">
+        <v>7.7896655604999996</v>
+      </c>
+      <c r="I5" s="1">
+        <v>9.1392076700000005E-2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1.50496271489999</v>
+      </c>
+      <c r="O5" s="1">
+        <v>5.7508319799999902E-2</v>
+      </c>
+      <c r="R5" s="1">
+        <v>8.0266894699999994E-2</v>
+      </c>
+      <c r="U5" s="1">
+        <v>0.14648018700000001</v>
+      </c>
+      <c r="X5" s="1">
+        <v>0.22424833150000001</v>
+      </c>
+      <c r="AA5" s="1">
+        <v>0.1457526992</v>
+      </c>
+      <c r="AD5" s="1">
+        <v>1.5127066299</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>1.93910095E-2</v>
+      </c>
+      <c r="AJ5" s="1">
+        <v>0.57490099240000003</v>
+      </c>
+      <c r="AM5" s="1">
+        <v>11.6087681536</v>
+      </c>
+    </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B14" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="T14" s="2"/>
     </row>
   </sheetData>
@@ -2207,4 +2264,578 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE3BDD0-3A87-544A-A16E-D142A4C1F8FB}">
+  <dimension ref="A1:O15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>2.0424912999999999E-2</v>
+      </c>
+      <c r="D5">
+        <v>7.7867697349999903</v>
+      </c>
+      <c r="E5">
+        <v>9.1322597999999894E-2</v>
+      </c>
+      <c r="F5">
+        <v>1.5043494099999899</v>
+      </c>
+      <c r="G5">
+        <v>5.7297887999999901E-2</v>
+      </c>
+      <c r="H5">
+        <v>8.0126062999999803E-2</v>
+      </c>
+      <c r="I5">
+        <v>0.14635807000000001</v>
+      </c>
+      <c r="J5">
+        <v>0.22410363699999999</v>
+      </c>
+      <c r="K5">
+        <v>0.145887511</v>
+      </c>
+      <c r="L5">
+        <v>1.5135437140000001</v>
+      </c>
+      <c r="M5">
+        <v>1.9270493999999899E-2</v>
+      </c>
+      <c r="N5">
+        <v>0.63718657899999998</v>
+      </c>
+      <c r="O5">
+        <v>11.605081670000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2.1145951E-2</v>
+      </c>
+      <c r="D6">
+        <v>7.7860681689999902</v>
+      </c>
+      <c r="E6">
+        <v>9.1019702999999993E-2</v>
+      </c>
+      <c r="F6">
+        <v>1.504760248</v>
+      </c>
+      <c r="G6">
+        <v>5.8056615999999998E-2</v>
+      </c>
+      <c r="H6">
+        <v>7.9142330999999899E-2</v>
+      </c>
+      <c r="I6">
+        <v>0.14721379100000001</v>
+      </c>
+      <c r="J6">
+        <v>0.22464350599999999</v>
+      </c>
+      <c r="K6">
+        <v>0.14654013999999899</v>
+      </c>
+      <c r="L6">
+        <v>1.5158264749999999</v>
+      </c>
+      <c r="M6">
+        <v>2.0120513999999999E-2</v>
+      </c>
+      <c r="N6">
+        <v>0.58061084600000001</v>
+      </c>
+      <c r="O6">
+        <v>11.611603560000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2.0321663E-2</v>
+      </c>
+      <c r="D7">
+        <v>7.7858370370000003</v>
+      </c>
+      <c r="E7">
+        <v>9.1435814000000198E-2</v>
+      </c>
+      <c r="F7">
+        <v>1.50463510299999</v>
+      </c>
+      <c r="G7">
+        <v>5.7139267999999903E-2</v>
+      </c>
+      <c r="H7">
+        <v>8.0468895999999998E-2</v>
+      </c>
+      <c r="I7">
+        <v>0.146477828</v>
+      </c>
+      <c r="J7">
+        <v>0.22378975800000001</v>
+      </c>
+      <c r="K7">
+        <v>0.14580547599999999</v>
+      </c>
+      <c r="L7">
+        <v>1.5118537869999999</v>
+      </c>
+      <c r="M7">
+        <v>1.9273346999999899E-2</v>
+      </c>
+      <c r="N7">
+        <v>0.56270112800000005</v>
+      </c>
+      <c r="O7">
+        <v>11.603158564999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>2.0864639000000001E-2</v>
+      </c>
+      <c r="D8">
+        <v>7.791942186</v>
+      </c>
+      <c r="E8">
+        <v>9.3432404999999899E-2</v>
+      </c>
+      <c r="F8">
+        <v>1.5056955270000001</v>
+      </c>
+      <c r="G8">
+        <v>5.7837718999999899E-2</v>
+      </c>
+      <c r="H8">
+        <v>8.0883411999999794E-2</v>
+      </c>
+      <c r="I8">
+        <v>0.14729577499999999</v>
+      </c>
+      <c r="J8">
+        <v>0.22659679099999999</v>
+      </c>
+      <c r="K8">
+        <v>0.14671094299999901</v>
+      </c>
+      <c r="L8">
+        <v>1.5164940629999999</v>
+      </c>
+      <c r="M8">
+        <v>1.9708712999999999E-2</v>
+      </c>
+      <c r="N8">
+        <v>0.56443909199999998</v>
+      </c>
+      <c r="O8">
+        <v>11.62344429</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>2.0280942999999899E-2</v>
+      </c>
+      <c r="D9">
+        <v>7.7999430569999904</v>
+      </c>
+      <c r="E9">
+        <v>9.0877374999999802E-2</v>
+      </c>
+      <c r="F9">
+        <v>1.50655010599999</v>
+      </c>
+      <c r="G9">
+        <v>5.7248313999999897E-2</v>
+      </c>
+      <c r="H9">
+        <v>8.0485838000000101E-2</v>
+      </c>
+      <c r="I9">
+        <v>0.14656117699999999</v>
+      </c>
+      <c r="J9">
+        <v>0.22409077799999999</v>
+      </c>
+      <c r="K9">
+        <v>0.14573356700000001</v>
+      </c>
+      <c r="L9">
+        <v>1.51249728199999</v>
+      </c>
+      <c r="M9">
+        <v>1.9202230000000001E-2</v>
+      </c>
+      <c r="N9">
+        <v>0.562185775</v>
+      </c>
+      <c r="O9">
+        <v>11.619479439999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>2.043876E-2</v>
+      </c>
+      <c r="D10">
+        <v>7.7974293039999996</v>
+      </c>
+      <c r="E10">
+        <v>9.1080436999999903E-2</v>
+      </c>
+      <c r="F10">
+        <v>1.5064454389999899</v>
+      </c>
+      <c r="G10">
+        <v>5.7185278999999797E-2</v>
+      </c>
+      <c r="H10">
+        <v>8.0402278999999993E-2</v>
+      </c>
+      <c r="I10">
+        <v>0.14645081199999899</v>
+      </c>
+      <c r="J10">
+        <v>0.22453524499999999</v>
+      </c>
+      <c r="K10">
+        <v>0.145886615999999</v>
+      </c>
+      <c r="L10">
+        <v>1.511602659</v>
+      </c>
+      <c r="M10">
+        <v>1.9318756999999999E-2</v>
+      </c>
+      <c r="N10">
+        <v>0.57984765400000005</v>
+      </c>
+      <c r="O10">
+        <v>11.616513956</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>2.0353184E-2</v>
+      </c>
+      <c r="D11">
+        <v>7.7924300309999897</v>
+      </c>
+      <c r="E11">
+        <v>9.0809097000000102E-2</v>
+      </c>
+      <c r="F11">
+        <v>1.5053146959999999</v>
+      </c>
+      <c r="G11">
+        <v>5.7189707999999902E-2</v>
+      </c>
+      <c r="H11">
+        <v>8.0279349E-2</v>
+      </c>
+      <c r="I11">
+        <v>0.146382653999999</v>
+      </c>
+      <c r="J11">
+        <v>0.22355650699999999</v>
+      </c>
+      <c r="K11">
+        <v>0.14538958199999999</v>
+      </c>
+      <c r="L11">
+        <v>1.513626312</v>
+      </c>
+      <c r="M11">
+        <v>1.9171847999999901E-2</v>
+      </c>
+      <c r="N11">
+        <v>0.560336846</v>
+      </c>
+      <c r="O11">
+        <v>11.610014887</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>2.0289628999999899E-2</v>
+      </c>
+      <c r="D12">
+        <v>7.7860702429999904</v>
+      </c>
+      <c r="E12">
+        <v>9.1088189E-2</v>
+      </c>
+      <c r="F12">
+        <v>1.5032416559999899</v>
+      </c>
+      <c r="G12">
+        <v>5.7050234999999901E-2</v>
+      </c>
+      <c r="H12">
+        <v>8.02704679999999E-2</v>
+      </c>
+      <c r="I12">
+        <v>0.14590045199999899</v>
+      </c>
+      <c r="J12">
+        <v>0.223113902999999</v>
+      </c>
+      <c r="K12">
+        <v>0.14498377500000001</v>
+      </c>
+      <c r="L12">
+        <v>1.51002137499999</v>
+      </c>
+      <c r="M12">
+        <v>1.9153499000000001E-2</v>
+      </c>
+      <c r="N12">
+        <v>0.56179270699999995</v>
+      </c>
+      <c r="O12">
+        <v>11.596820626</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>2.03218539999999E-2</v>
+      </c>
+      <c r="D13">
+        <v>7.7836237120000096</v>
+      </c>
+      <c r="E13">
+        <v>9.1111495999999903E-2</v>
+      </c>
+      <c r="F13">
+        <v>1.5051262249999999</v>
+      </c>
+      <c r="G13">
+        <v>5.7253967999999898E-2</v>
+      </c>
+      <c r="H13">
+        <v>8.0286094000000099E-2</v>
+      </c>
+      <c r="I13">
+        <v>0.145972402</v>
+      </c>
+      <c r="J13">
+        <v>0.22355931900000001</v>
+      </c>
+      <c r="K13">
+        <v>0.145110973999999</v>
+      </c>
+      <c r="L13">
+        <v>1.511406241</v>
+      </c>
+      <c r="M13">
+        <v>1.9221361999999999E-2</v>
+      </c>
+      <c r="N13">
+        <v>0.58119497399999998</v>
+      </c>
+      <c r="O13">
+        <v>11.598596659</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>2.04681699999999E-2</v>
+      </c>
+      <c r="D14">
+        <v>7.786542131</v>
+      </c>
+      <c r="E14">
+        <v>9.1743652999999897E-2</v>
+      </c>
+      <c r="F14">
+        <v>1.5035087389999899</v>
+      </c>
+      <c r="G14">
+        <v>5.8824202999999797E-2</v>
+      </c>
+      <c r="H14">
+        <v>8.0324217000000003E-2</v>
+      </c>
+      <c r="I14">
+        <v>0.14618890900000001</v>
+      </c>
+      <c r="J14">
+        <v>0.22449387100000001</v>
+      </c>
+      <c r="K14">
+        <v>0.145478408</v>
+      </c>
+      <c r="L14">
+        <v>1.510194391</v>
+      </c>
+      <c r="M14">
+        <v>1.9469330999999999E-2</v>
+      </c>
+      <c r="N14">
+        <v>0.55871432300000001</v>
+      </c>
+      <c r="O14">
+        <v>11.602967883</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2.0490970599999998E-2</v>
+      </c>
+      <c r="D15" s="1">
+        <v>7.7896655604999996</v>
+      </c>
+      <c r="E15" s="1">
+        <v>9.1392076700000005E-2</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1.50496271489999</v>
+      </c>
+      <c r="G15" s="1">
+        <v>5.7508319799999902E-2</v>
+      </c>
+      <c r="H15" s="1">
+        <v>8.0266894699999994E-2</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0.14648018700000001</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.22424833150000001</v>
+      </c>
+      <c r="K15" s="1">
+        <v>0.1457526992</v>
+      </c>
+      <c r="L15" s="1">
+        <v>1.5127066299</v>
+      </c>
+      <c r="M15" s="1">
+        <v>1.93910095E-2</v>
+      </c>
+      <c r="N15" s="1">
+        <v>0.57490099240000003</v>
+      </c>
+      <c r="O15" s="1">
+        <v>11.6087681536</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:O3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Complete initial analysis worksheet
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA1CDE0-9160-0642-80B2-BA4607FE6B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05EABA7-3707-E845-95BC-AFF0085B4065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43100" yWindow="1360" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
+    <workbookView xWindow="33400" yWindow="660" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_Results" sheetId="1" r:id="rId1"/>
     <sheet name="Trackslot_Xorwow" sheetId="2" r:id="rId2"/>
     <sheet name="Trackslot_Ranluxpp" sheetId="3" r:id="rId3"/>
     <sheet name="Track_Xorwow" sheetId="4" r:id="rId4"/>
+    <sheet name="Track_Ranluxpp" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="26">
   <si>
     <t>Branch</t>
   </si>
@@ -907,50 +908,253 @@
       <c r="B5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>2.0490970599999998E-2</v>
       </c>
-      <c r="F5" s="1">
+      <c r="D5" s="2">
+        <v>2.16922599E-2</v>
+      </c>
+      <c r="E5">
+        <f>((C5-D5)/C5)*100</f>
+        <v>-5.8625300062653052</v>
+      </c>
+      <c r="F5" s="2">
         <v>7.7896655604999996</v>
       </c>
-      <c r="I5" s="1">
+      <c r="G5" s="2">
+        <v>7.7896106538999899</v>
+      </c>
+      <c r="H5" s="2">
+        <f>((F5-G5)/F5)*100</f>
+        <v>7.0486466438496851E-4</v>
+      </c>
+      <c r="I5" s="2">
         <v>9.1392076700000005E-2</v>
       </c>
-      <c r="L5" s="1">
+      <c r="J5" s="2">
+        <v>9.8359574300000002E-2</v>
+      </c>
+      <c r="K5">
+        <f>((I5-J5)/I5)*100</f>
+        <v>-7.6237436018345743</v>
+      </c>
+      <c r="L5" s="2">
         <v>1.50496271489999</v>
       </c>
-      <c r="O5" s="1">
+      <c r="M5" s="2">
+        <v>1.51386815239999</v>
+      </c>
+      <c r="N5">
+        <f>((L5-M5)/L5)*100</f>
+        <v>-0.59173808173657938</v>
+      </c>
+      <c r="O5" s="2">
         <v>5.7508319799999902E-2</v>
       </c>
-      <c r="R5" s="1">
+      <c r="P5" s="2">
+        <v>5.6594890299999999E-2</v>
+      </c>
+      <c r="Q5">
+        <f>((O5-P5)/O5)*100</f>
+        <v>1.5883432226442902</v>
+      </c>
+      <c r="R5" s="2">
         <v>8.0266894699999994E-2</v>
       </c>
-      <c r="U5" s="1">
+      <c r="S5" s="2">
+        <v>0.45789087749999902</v>
+      </c>
+      <c r="T5">
+        <f>((R5-S5)/R5)*100</f>
+        <v>-470.46043603827002</v>
+      </c>
+      <c r="U5" s="2">
         <v>0.14648018700000001</v>
       </c>
-      <c r="X5" s="1">
+      <c r="V5" s="2">
+        <v>6.0640335470000002</v>
+      </c>
+      <c r="W5">
+        <f>((U5-V5)/U5)*100</f>
+        <v>-4039.83192621129</v>
+      </c>
+      <c r="X5" s="2">
         <v>0.22424833150000001</v>
       </c>
-      <c r="AA5" s="1">
+      <c r="Y5" s="2">
+        <v>0.27265967940000002</v>
+      </c>
+      <c r="Z5">
+        <f>((X5-Y5)/X5)*100</f>
+        <v>-21.588275630046329</v>
+      </c>
+      <c r="AA5" s="2">
         <v>0.1457526992</v>
       </c>
-      <c r="AD5" s="1">
+      <c r="AB5" s="2">
+        <v>0.49234086289999901</v>
+      </c>
+      <c r="AC5">
+        <f>((AA5-AB5)/AA5)*100</f>
+        <v>-237.79193497090242</v>
+      </c>
+      <c r="AD5" s="2">
         <v>1.5127066299</v>
       </c>
-      <c r="AG5" s="1">
+      <c r="AE5" s="2">
+        <v>3.9051250898999901</v>
+      </c>
+      <c r="AF5">
+        <f>((AD5-AE5)/AD5)*100</f>
+        <v>-158.154820816654</v>
+      </c>
+      <c r="AG5" s="2">
         <v>1.93910095E-2</v>
       </c>
-      <c r="AJ5" s="1">
+      <c r="AH5" s="2">
+        <v>2.0148734299999999E-2</v>
+      </c>
+      <c r="AI5">
+        <f>((AG5-AH5)/AG5)*100</f>
+        <v>-3.9076088328459537</v>
+      </c>
+      <c r="AJ5" s="2">
         <v>0.57490099240000003</v>
       </c>
-      <c r="AM5" s="1">
+      <c r="AK5" s="2">
+        <v>0.55649489640000005</v>
+      </c>
+      <c r="AL5">
+        <f>((AJ5-AK5)/AJ5)*100</f>
+        <v>3.2016114502014177</v>
+      </c>
+      <c r="AM5" s="2">
         <v>11.6087681536</v>
       </c>
+      <c r="AN5" s="2">
+        <v>20.709697601799999</v>
+      </c>
+      <c r="AO5">
+        <f>((AM5-AN5)/AM5)*100</f>
+        <v>-78.397029967195152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <f>((C4-C5)/C4)*100</f>
+        <v>99.567349813285759</v>
+      </c>
+      <c r="D6">
+        <f>((D4-D5)/D4)*100</f>
+        <v>-0.1156244995177548</v>
+      </c>
+      <c r="F6">
+        <f>((F4-F5)/F4)*100</f>
+        <v>63.222711162142488</v>
+      </c>
+      <c r="G6">
+        <f>((G4-G5)/G4)*100</f>
+        <v>1.4856356759473173E-2</v>
+      </c>
+      <c r="I6">
+        <f>((I4-I5)/I4)*100</f>
+        <v>99.033107888925528</v>
+      </c>
+      <c r="J6">
+        <f>((J4-J5)/J4)*100</f>
+        <v>0.50763629045109337</v>
+      </c>
+      <c r="L6">
+        <f>((L4-L5)/L4)*100</f>
+        <v>75.823827539543657</v>
+      </c>
+      <c r="M6">
+        <f>((M4-M5)/M4)*100</f>
+        <v>1.8275331902369348E-2</v>
+      </c>
+      <c r="O6">
+        <f>((O4-O5)/O4)*100</f>
+        <v>98.794366694351481</v>
+      </c>
+      <c r="P6">
+        <f>((P4-P5)/P4)*100</f>
+        <v>-1.53383657642925E-2</v>
+      </c>
+      <c r="R6">
+        <f>((R4-R5)/R4)*100</f>
+        <v>98.323548909138765</v>
+      </c>
+      <c r="S6">
+        <f>((S4-S5)/S4)*100</f>
+        <v>-3.9150816714984731E-3</v>
+      </c>
+      <c r="U6">
+        <f>((U4-U5)/U4)*100</f>
+        <v>96.983588313420526</v>
+      </c>
+      <c r="V6">
+        <f>((V4-V5)/V4)*100</f>
+        <v>5.2696881875534066E-3</v>
+      </c>
+      <c r="X6">
+        <f>((X4-X5)/X4)*100</f>
+        <v>95.465851086659754</v>
+      </c>
+      <c r="Y6">
+        <f>((Y4-Y5)/Y4)*100</f>
+        <v>-6.6165150331572747E-2</v>
+      </c>
+      <c r="AA6">
+        <f>((AA4-AA5)/AA4)*100</f>
+        <v>96.994229968320994</v>
+      </c>
+      <c r="AB6">
+        <f>((AB4-AB5)/AB4)*100</f>
+        <v>9.3652964459275539E-3</v>
+      </c>
+      <c r="AD6">
+        <f>((AD4-AD5)/AD4)*100</f>
+        <v>85.441885192023463</v>
+      </c>
+      <c r="AE6">
+        <f>((AE4-AE5)/AE4)*100</f>
+        <v>-2.2412488665593273E-2</v>
+      </c>
+      <c r="AG6">
+        <f>((AG4-AG5)/AG4)*100</f>
+        <v>99.590207870875858</v>
+      </c>
+      <c r="AH6">
+        <f>((AH4-AH5)/AH4)*100</f>
+        <v>-4.0182434508662906E-2</v>
+      </c>
+      <c r="AJ6">
+        <f>((AJ4-AJ5)/AJ4)*100</f>
+        <v>-1.9379795505074249</v>
+      </c>
+      <c r="AK6">
+        <f>((AK4-AK5)/AK4)*100</f>
+        <v>0.62771900991408691</v>
+      </c>
+      <c r="AM6">
+        <f>((AM4-AM5)/AM4)*100</f>
+        <v>85.659713516429363</v>
+      </c>
+      <c r="AN6">
+        <f>((AN4-AN5)/AN4)*100</f>
+        <v>5.3476771764439362E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="B14" s="1"/>
       <c r="T14" s="2"/>
     </row>
   </sheetData>
@@ -970,8 +1174,8 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:T2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4">
-    <cfRule type="colorScale" priority="14">
+  <conditionalFormatting sqref="E4:E5">
+    <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -980,8 +1184,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4">
-    <cfRule type="colorScale" priority="12">
+  <conditionalFormatting sqref="H4:H5">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -990,8 +1194,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4">
-    <cfRule type="colorScale" priority="11">
+  <conditionalFormatting sqref="K4:K5">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1000,8 +1204,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N4">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="N4:N5">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1010,8 +1214,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q4">
-    <cfRule type="colorScale" priority="9">
+  <conditionalFormatting sqref="Q4:Q5">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1020,8 +1224,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T4">
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="T4:T5">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1030,8 +1234,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W4">
-    <cfRule type="colorScale" priority="7">
+  <conditionalFormatting sqref="W4:W5">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1040,8 +1244,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z4">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="Z4:Z5">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1050,8 +1254,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="AC4:AC5">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1060,8 +1264,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF4">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="AF4:AF5">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1070,8 +1274,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI4">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="AI4:AI5">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1080,8 +1284,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL4">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="AL4:AL5">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1090,12 +1294,142 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AO4">
+  <conditionalFormatting sqref="AO4:AO5">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:D6">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F6:G6">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:J6">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6:M6">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O6:P6">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R6:S6">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U6:V6">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X6:Y6">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6:AB6">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD6:AE6">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG6:AH6">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ6:AK6">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM6:AN6">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
+        <color rgb="FFFF0000"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
@@ -2838,4 +3172,578 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBF611A7-FF5C-9946-82AC-26D645B98B8C}">
+  <dimension ref="A1:O15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>2.1670388999999901E-2</v>
+      </c>
+      <c r="D5">
+        <v>7.788605767</v>
+      </c>
+      <c r="E5">
+        <v>9.9566999999999795E-2</v>
+      </c>
+      <c r="F5">
+        <v>1.51476287599999</v>
+      </c>
+      <c r="G5">
+        <v>5.6594470000000001E-2</v>
+      </c>
+      <c r="H5">
+        <v>0.45763494700000001</v>
+      </c>
+      <c r="I5">
+        <v>6.0642653989999999</v>
+      </c>
+      <c r="J5">
+        <v>0.27255439599999898</v>
+      </c>
+      <c r="K5">
+        <v>0.49231615699999998</v>
+      </c>
+      <c r="L5">
+        <v>3.9079429750000001</v>
+      </c>
+      <c r="M5">
+        <v>2.0160246999999999E-2</v>
+      </c>
+      <c r="N5">
+        <v>0.62630026999999999</v>
+      </c>
+      <c r="O5">
+        <v>20.713497519000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2.19130099999999E-2</v>
+      </c>
+      <c r="D6">
+        <v>7.79280851900001</v>
+      </c>
+      <c r="E6">
+        <v>9.9675741000000095E-2</v>
+      </c>
+      <c r="F6">
+        <v>1.514690286</v>
+      </c>
+      <c r="G6">
+        <v>5.6976826000000001E-2</v>
+      </c>
+      <c r="H6">
+        <v>0.45819648799999901</v>
+      </c>
+      <c r="I6">
+        <v>6.0626823300000003</v>
+      </c>
+      <c r="J6">
+        <v>0.274515538</v>
+      </c>
+      <c r="K6">
+        <v>0.49315212899999999</v>
+      </c>
+      <c r="L6">
+        <v>3.900064135</v>
+      </c>
+      <c r="M6">
+        <v>2.0464525000000001E-2</v>
+      </c>
+      <c r="N6">
+        <v>0.54645062600000005</v>
+      </c>
+      <c r="O6">
+        <v>20.712612427</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2.1715781E-2</v>
+      </c>
+      <c r="D7">
+        <v>7.78769075099998</v>
+      </c>
+      <c r="E7">
+        <v>9.8289989999999897E-2</v>
+      </c>
+      <c r="F7">
+        <v>1.51437557399999</v>
+      </c>
+      <c r="G7">
+        <v>5.6514841000000003E-2</v>
+      </c>
+      <c r="H7">
+        <v>0.45803918399999999</v>
+      </c>
+      <c r="I7">
+        <v>6.0630073089999899</v>
+      </c>
+      <c r="J7">
+        <v>0.27229793999999902</v>
+      </c>
+      <c r="K7">
+        <v>0.49229077099999902</v>
+      </c>
+      <c r="L7">
+        <v>3.9083897669999899</v>
+      </c>
+      <c r="M7">
+        <v>2.0096164E-2</v>
+      </c>
+      <c r="N7">
+        <v>0.54734508500000001</v>
+      </c>
+      <c r="O7">
+        <v>20.709862891</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>2.1558777000000001E-2</v>
+      </c>
+      <c r="D8">
+        <v>7.7885421700000004</v>
+      </c>
+      <c r="E8">
+        <v>9.7385553000000097E-2</v>
+      </c>
+      <c r="F8">
+        <v>1.5140554819999901</v>
+      </c>
+      <c r="G8">
+        <v>5.6435298999999897E-2</v>
+      </c>
+      <c r="H8">
+        <v>0.45793884199999901</v>
+      </c>
+      <c r="I8">
+        <v>6.064377371</v>
+      </c>
+      <c r="J8">
+        <v>0.27229752899999998</v>
+      </c>
+      <c r="K8">
+        <v>0.492120908999999</v>
+      </c>
+      <c r="L8">
+        <v>3.9084012960000001</v>
+      </c>
+      <c r="M8">
+        <v>1.9987675999999999E-2</v>
+      </c>
+      <c r="N8">
+        <v>0.55720628400000005</v>
+      </c>
+      <c r="O8">
+        <v>20.710153963</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>2.1566398000000001E-2</v>
+      </c>
+      <c r="D9">
+        <v>7.7886827629999997</v>
+      </c>
+      <c r="E9">
+        <v>9.7693707000000005E-2</v>
+      </c>
+      <c r="F9">
+        <v>1.5148509079999899</v>
+      </c>
+      <c r="G9">
+        <v>5.6489028999999899E-2</v>
+      </c>
+      <c r="H9">
+        <v>0.45799976599999997</v>
+      </c>
+      <c r="I9">
+        <v>6.0669434850000004</v>
+      </c>
+      <c r="J9">
+        <v>0.27245112300000002</v>
+      </c>
+      <c r="K9">
+        <v>0.49225550400000001</v>
+      </c>
+      <c r="L9">
+        <v>3.9067603819999901</v>
+      </c>
+      <c r="M9">
+        <v>2.00978629999999E-2</v>
+      </c>
+      <c r="N9">
+        <v>0.54859861300000001</v>
+      </c>
+      <c r="O9">
+        <v>20.713437281000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>2.1632118999999901E-2</v>
+      </c>
+      <c r="D10">
+        <v>7.7915927429999901</v>
+      </c>
+      <c r="E10">
+        <v>9.7113913000000093E-2</v>
+      </c>
+      <c r="F10">
+        <v>1.51434344799999</v>
+      </c>
+      <c r="G10">
+        <v>5.64154830000001E-2</v>
+      </c>
+      <c r="H10">
+        <v>0.45765355000000002</v>
+      </c>
+      <c r="I10">
+        <v>6.0666592069999998</v>
+      </c>
+      <c r="J10">
+        <v>0.271916721999999</v>
+      </c>
+      <c r="K10">
+        <v>0.493578724999999</v>
+      </c>
+      <c r="L10">
+        <v>3.90671174799999</v>
+      </c>
+      <c r="M10">
+        <v>2.0044738999999999E-2</v>
+      </c>
+      <c r="N10">
+        <v>0.54808315500000004</v>
+      </c>
+      <c r="O10">
+        <v>20.715232767</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>2.1658759999999899E-2</v>
+      </c>
+      <c r="D11">
+        <v>7.7947981879999997</v>
+      </c>
+      <c r="E11">
+        <v>9.8980616000000105E-2</v>
+      </c>
+      <c r="F11">
+        <v>1.5148128999999999</v>
+      </c>
+      <c r="G11">
+        <v>5.6672052000000001E-2</v>
+      </c>
+      <c r="H11">
+        <v>0.457924215999999</v>
+      </c>
+      <c r="I11">
+        <v>6.0668586840000103</v>
+      </c>
+      <c r="J11">
+        <v>0.272893575</v>
+      </c>
+      <c r="K11">
+        <v>0.492327072999999</v>
+      </c>
+      <c r="L11">
+        <v>3.9048722989999902</v>
+      </c>
+      <c r="M11">
+        <v>2.0216452999999999E-2</v>
+      </c>
+      <c r="N11">
+        <v>0.54761473100000002</v>
+      </c>
+      <c r="O11">
+        <v>20.719440948999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>2.1639038999999999E-2</v>
+      </c>
+      <c r="D12">
+        <v>7.7899716459999997</v>
+      </c>
+      <c r="E12">
+        <v>9.8083506999999903E-2</v>
+      </c>
+      <c r="F12">
+        <v>1.5127594169999901</v>
+      </c>
+      <c r="G12">
+        <v>5.6608270000000002E-2</v>
+      </c>
+      <c r="H12">
+        <v>0.45777858199999899</v>
+      </c>
+      <c r="I12">
+        <v>6.0622548540000096</v>
+      </c>
+      <c r="J12">
+        <v>0.27232184799999998</v>
+      </c>
+      <c r="K12">
+        <v>0.49182620599999899</v>
+      </c>
+      <c r="L12">
+        <v>3.9037054969999998</v>
+      </c>
+      <c r="M12">
+        <v>2.0026265000000001E-2</v>
+      </c>
+      <c r="N12">
+        <v>0.54539367400000005</v>
+      </c>
+      <c r="O12">
+        <v>20.704204261000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>2.1713296999999999E-2</v>
+      </c>
+      <c r="D13">
+        <v>7.787347113</v>
+      </c>
+      <c r="E13">
+        <v>9.7883269000000106E-2</v>
+      </c>
+      <c r="F13">
+        <v>1.51182173999999</v>
+      </c>
+      <c r="G13">
+        <v>5.6496790999999998E-2</v>
+      </c>
+      <c r="H13">
+        <v>0.45767707799999902</v>
+      </c>
+      <c r="I13">
+        <v>6.0607472580000001</v>
+      </c>
+      <c r="J13">
+        <v>0.27223769999999903</v>
+      </c>
+      <c r="K13">
+        <v>0.49176235600000001</v>
+      </c>
+      <c r="L13">
+        <v>3.89744741999999</v>
+      </c>
+      <c r="M13">
+        <v>2.0108869000000001E-2</v>
+      </c>
+      <c r="N13">
+        <v>0.55015700700000003</v>
+      </c>
+      <c r="O13">
+        <v>20.692585380000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>2.1855028999999901E-2</v>
+      </c>
+      <c r="D14">
+        <v>7.7860668789999696</v>
+      </c>
+      <c r="E14">
+        <v>9.8922446999999997E-2</v>
+      </c>
+      <c r="F14">
+        <v>1.51220889299999</v>
+      </c>
+      <c r="G14">
+        <v>5.6745841999999901E-2</v>
+      </c>
+      <c r="H14">
+        <v>0.45806612199999902</v>
+      </c>
+      <c r="I14">
+        <v>6.0625395729999996</v>
+      </c>
+      <c r="J14">
+        <v>0.27311042299999999</v>
+      </c>
+      <c r="K14">
+        <v>0.49177879899999999</v>
+      </c>
+      <c r="L14">
+        <v>3.9069553799999999</v>
+      </c>
+      <c r="M14">
+        <v>2.0284541999999999E-2</v>
+      </c>
+      <c r="N14">
+        <v>0.54779951900000001</v>
+      </c>
+      <c r="O14">
+        <v>20.705948580000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2.16922599E-2</v>
+      </c>
+      <c r="D15" s="1">
+        <v>7.7896106538999899</v>
+      </c>
+      <c r="E15" s="1">
+        <v>9.8359574300000002E-2</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1.51386815239999</v>
+      </c>
+      <c r="G15" s="1">
+        <v>5.6594890299999999E-2</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0.45789087749999902</v>
+      </c>
+      <c r="I15" s="1">
+        <v>6.0640335470000002</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.27265967940000002</v>
+      </c>
+      <c r="K15" s="1">
+        <v>0.49234086289999901</v>
+      </c>
+      <c r="L15" s="1">
+        <v>3.9051250898999901</v>
+      </c>
+      <c r="M15" s="1">
+        <v>2.0148734299999999E-2</v>
+      </c>
+      <c r="N15" s="1">
+        <v>0.55649489640000005</v>
+      </c>
+      <c r="O15" s="1">
+        <v>20.709697601799999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:O3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Complete initial Dune analysis
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05EABA7-3707-E845-95BC-AFF0085B4065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F29E3D8-7825-7447-8785-B14548994AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33400" yWindow="660" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
+    <workbookView xWindow="56320" yWindow="0" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_Results" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="26">
   <si>
     <t>Branch</t>
   </si>
@@ -520,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B71848BA-D8C3-7041-A0EE-B663A4811CD2}">
-  <dimension ref="A1:AO14"/>
+  <dimension ref="A1:AO19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="42.1640625" bestFit="1" customWidth="1"/>
@@ -774,134 +774,134 @@
         <v>24</v>
       </c>
       <c r="C4" s="2">
-        <v>4.7361520297999897</v>
+        <v>2.10134848999999E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>2.1667207299999901E-2</v>
+        <v>2.1044281399999899E-2</v>
       </c>
       <c r="E4">
         <f>((C4-D4)/C4)*100</f>
-        <v>99.542514531550736</v>
+        <v>-0.14655589087938234</v>
       </c>
       <c r="F4" s="2">
-        <v>21.1806411148</v>
+        <v>7.7868371409000003</v>
       </c>
       <c r="G4" s="2">
-        <v>7.7907680781999904</v>
+        <v>7.7882990942999903</v>
       </c>
       <c r="H4">
         <f>((F4-G4)/F4)*100</f>
-        <v>63.217505853700615</v>
+        <v>-1.8774675436720758E-2</v>
       </c>
       <c r="I4" s="2">
-        <v>9.4521483475999908</v>
+        <v>0.10106857869999999</v>
       </c>
       <c r="J4" s="2">
-        <v>9.8861430799999997E-2</v>
+        <v>0.1008018878</v>
       </c>
       <c r="K4">
         <f>((I4-J4)/I4)*100</f>
-        <v>98.954085069717493</v>
+        <v>0.26387122825938303</v>
       </c>
       <c r="L4" s="2">
-        <v>6.2249833689000003</v>
+        <v>1.5133286373999999</v>
       </c>
       <c r="M4" s="2">
-        <v>1.51414486739999</v>
+        <v>1.5134209893999899</v>
       </c>
       <c r="N4">
         <f>((L4-M4)/L4)*100</f>
-        <v>75.67632268762911</v>
+        <v>-6.102574001949284E-3</v>
       </c>
       <c r="O4" s="2">
-        <v>4.7699677447999997</v>
+        <v>5.5878251300000001E-2</v>
       </c>
       <c r="P4" s="2">
-        <v>5.6586210900000003E-2</v>
+        <v>5.5854686299999998E-2</v>
       </c>
       <c r="Q4">
         <f>((O4-P4)/O4)*100</f>
-        <v>98.813698248553408</v>
+        <v>4.2172042703138721E-2</v>
       </c>
       <c r="R4" s="2">
-        <v>4.7879055426999999</v>
+        <v>0.45890807779999998</v>
       </c>
       <c r="S4" s="2">
-        <v>0.45787295140000001</v>
+        <v>0.45886056159999999</v>
       </c>
       <c r="T4">
         <f>((R4-S4)/R4)*100</f>
-        <v>90.436884200898504</v>
+        <v>1.0354186883738974E-2</v>
       </c>
       <c r="U4" s="2">
-        <v>4.8561072632000002</v>
+        <v>6.0628989352999998</v>
       </c>
       <c r="V4" s="2">
-        <v>6.06435311949999</v>
+        <v>6.0622900875000001</v>
       </c>
       <c r="W4">
         <f>((U4-V4)/U4)*100</f>
-        <v>-24.880954863912937</v>
+        <v>1.0042189495437705E-2</v>
       </c>
       <c r="X4" s="2">
-        <v>4.9457645918999997</v>
+        <v>0.27203544940000002</v>
       </c>
       <c r="Y4" s="2">
-        <v>0.27247939299999901</v>
+        <v>0.27205333569999901</v>
       </c>
       <c r="Z4">
         <f>((X4-Y4)/X4)*100</f>
-        <v>94.490651790296354</v>
+        <v>-6.5749886782926767E-3</v>
       </c>
       <c r="AA4" s="2">
-        <v>4.8490968258999896</v>
+        <v>0.49175476299999998</v>
       </c>
       <c r="AB4" s="2">
-        <v>0.49238697640000001</v>
+        <v>0.49182936509999903</v>
       </c>
       <c r="AC4">
         <f>((AA4-AB4)/AA4)*100</f>
-        <v>89.845800278310321</v>
+        <v>-1.5170590223453264E-2</v>
       </c>
       <c r="AD4" s="2">
-        <v>10.3908139883</v>
+        <v>3.9014598262999902</v>
       </c>
       <c r="AE4" s="2">
-        <v>3.9042500502999902</v>
+        <v>3.9008079268000002</v>
       </c>
       <c r="AF4">
         <f>((AD4-AE4)/AD4)*100</f>
-        <v>62.425946083760579</v>
+        <v>1.6709117330787542E-2</v>
       </c>
       <c r="AG4" s="2">
-        <v>4.7319136024999997</v>
+        <v>1.93700037999999E-2</v>
       </c>
       <c r="AH4" s="2">
-        <v>2.0140641300000001E-2</v>
+        <v>1.93747672E-2</v>
       </c>
       <c r="AI4">
         <f>((AG4-AH4)/AG4)*100</f>
-        <v>99.574365827614457</v>
+        <v>-2.459163172750858E-2</v>
       </c>
       <c r="AJ4" s="2">
-        <v>0.56397134309999997</v>
+        <v>0.54875180800000001</v>
       </c>
       <c r="AK4" s="2">
-        <v>0.56001018679999903</v>
+        <v>0.54884408070000001</v>
       </c>
       <c r="AL4">
         <f>((AJ4-AK4)/AJ4)*100</f>
-        <v>0.70236836471646147</v>
+        <v>-1.6815015213582085E-2</v>
       </c>
       <c r="AM4" s="2">
-        <v>80.952135558099997</v>
+        <v>20.700766578500001</v>
       </c>
       <c r="AN4" s="2">
-        <v>20.710805148799999</v>
+        <v>20.7009069424</v>
       </c>
       <c r="AO4">
         <f>((AM4-AN4)/AM4)*100</f>
-        <v>74.415986674081395</v>
+        <v>-6.7806136292530817E-4</v>
       </c>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.2">
@@ -909,134 +909,134 @@
         <v>25</v>
       </c>
       <c r="C5" s="2">
-        <v>2.0490970599999998E-2</v>
+        <v>2.1148022799999899E-2</v>
       </c>
       <c r="D5" s="2">
-        <v>2.16922599E-2</v>
+        <v>2.1138030700000001E-2</v>
       </c>
       <c r="E5">
         <f>((C5-D5)/C5)*100</f>
-        <v>-5.8625300062653052</v>
+        <v>4.7248388629019415E-2</v>
       </c>
       <c r="F5" s="2">
-        <v>7.7896655604999996</v>
+        <v>7.7888443829999998</v>
       </c>
       <c r="G5" s="2">
-        <v>7.7896106538999899</v>
-      </c>
-      <c r="H5" s="2">
+        <v>7.7902623423999904</v>
+      </c>
+      <c r="H5">
         <f>((F5-G5)/F5)*100</f>
-        <v>7.0486466438496851E-4</v>
+        <v>-1.8205003595724873E-2</v>
       </c>
       <c r="I5" s="2">
-        <v>9.1392076700000005E-2</v>
+        <v>0.1013372595</v>
       </c>
       <c r="J5" s="2">
-        <v>9.8359574300000002E-2</v>
+        <v>0.1010922164</v>
       </c>
       <c r="K5">
         <f>((I5-J5)/I5)*100</f>
-        <v>-7.6237436018345743</v>
+        <v>0.2418094797600035</v>
       </c>
       <c r="L5" s="2">
-        <v>1.50496271489999</v>
+        <v>1.5131773657000001</v>
       </c>
       <c r="M5" s="2">
-        <v>1.51386815239999</v>
+        <v>1.5147833314000001</v>
       </c>
       <c r="N5">
         <f>((L5-M5)/L5)*100</f>
-        <v>-0.59173808173657938</v>
+        <v>-0.10613201970921107</v>
       </c>
       <c r="O5" s="2">
-        <v>5.7508319799999902E-2</v>
+        <v>5.5961258899999998E-2</v>
       </c>
       <c r="P5" s="2">
-        <v>5.6594890299999999E-2</v>
+        <v>5.59714298E-2</v>
       </c>
       <c r="Q5">
         <f>((O5-P5)/O5)*100</f>
-        <v>1.5883432226442902</v>
+        <v>-1.8174894918244817E-2</v>
       </c>
       <c r="R5" s="2">
-        <v>8.0266894699999994E-2</v>
+        <v>0.45887892660000001</v>
       </c>
       <c r="S5" s="2">
-        <v>0.45789087749999902</v>
+        <v>0.45877713409999998</v>
       </c>
       <c r="T5">
         <f>((R5-S5)/R5)*100</f>
-        <v>-470.46043603827002</v>
+        <v>2.2182866568802424E-2</v>
       </c>
       <c r="U5" s="2">
-        <v>0.14648018700000001</v>
+        <v>6.0627548560999998</v>
       </c>
       <c r="V5" s="2">
-        <v>6.0640335470000002</v>
+        <v>6.0636236880999999</v>
       </c>
       <c r="W5">
         <f>((U5-V5)/U5)*100</f>
-        <v>-4039.83192621129</v>
+        <v>-1.4330647051083181E-2</v>
       </c>
       <c r="X5" s="2">
-        <v>0.22424833150000001</v>
+        <v>0.27224948490000001</v>
       </c>
       <c r="Y5" s="2">
-        <v>0.27265967940000002</v>
+        <v>0.27250950699999998</v>
       </c>
       <c r="Z5">
         <f>((X5-Y5)/X5)*100</f>
-        <v>-21.588275630046329</v>
+        <v>-9.5508757379463141E-2</v>
       </c>
       <c r="AA5" s="2">
-        <v>0.1457526992</v>
+        <v>0.49188873370000002</v>
       </c>
       <c r="AB5" s="2">
-        <v>0.49234086289999901</v>
+        <v>0.49214803059999901</v>
       </c>
       <c r="AC5">
         <f>((AA5-AB5)/AA5)*100</f>
-        <v>-237.79193497090242</v>
+        <v>-5.2714543398574322E-2</v>
       </c>
       <c r="AD5" s="2">
-        <v>1.5127066299</v>
+        <v>3.8996550481000001</v>
       </c>
       <c r="AE5" s="2">
-        <v>3.9051250898999901</v>
+        <v>3.8996497178</v>
       </c>
       <c r="AF5">
         <f>((AD5-AE5)/AD5)*100</f>
-        <v>-158.154820816654</v>
+        <v>1.3668644878339834E-4</v>
       </c>
       <c r="AG5" s="2">
-        <v>1.93910095E-2</v>
+        <v>1.9472640100000001E-2</v>
       </c>
       <c r="AH5" s="2">
-        <v>2.0148734299999999E-2</v>
+        <v>1.9451079699999999E-2</v>
       </c>
       <c r="AI5">
         <f>((AG5-AH5)/AG5)*100</f>
-        <v>-3.9076088328459537</v>
+        <v>0.11072150406560535</v>
       </c>
       <c r="AJ5" s="2">
-        <v>0.57490099240000003</v>
+        <v>0.55042533940000005</v>
       </c>
       <c r="AK5" s="2">
-        <v>0.55649489640000005</v>
+        <v>0.55477528669999998</v>
       </c>
       <c r="AL5">
         <f>((AJ5-AK5)/AJ5)*100</f>
-        <v>3.2016114502014177</v>
+        <v>-0.7902883440543752</v>
       </c>
       <c r="AM5" s="2">
-        <v>11.6087681536</v>
+        <v>20.701861121499999</v>
       </c>
       <c r="AN5" s="2">
-        <v>20.709697601799999</v>
+        <v>20.705847007199999</v>
       </c>
       <c r="AO5">
         <f>((AM5-AN5)/AM5)*100</f>
-        <v>-78.397029967195152</v>
+        <v>-1.9253755382703359E-2</v>
       </c>
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.2">
@@ -1045,117 +1045,127 @@
       </c>
       <c r="C6">
         <f>((C4-C5)/C4)*100</f>
-        <v>99.567349813285759</v>
+        <v>-0.64024554061472838</v>
       </c>
       <c r="D6">
         <f>((D4-D5)/D4)*100</f>
-        <v>-0.1156244995177548</v>
+        <v>-0.44548586962015346</v>
       </c>
       <c r="F6">
         <f>((F4-F5)/F4)*100</f>
-        <v>63.222711162142488</v>
+        <v>-2.5777373581585869E-2</v>
       </c>
       <c r="G6">
         <f>((G4-G5)/G4)*100</f>
-        <v>1.4856356759473173E-2</v>
+        <v>-2.5207661855678808E-2</v>
       </c>
       <c r="I6">
         <f>((I4-I5)/I4)*100</f>
-        <v>99.033107888925528</v>
+        <v>-0.26584008942831217</v>
       </c>
       <c r="J6">
         <f>((J4-J5)/J4)*100</f>
-        <v>0.50763629045109337</v>
+        <v>-0.28801901069158398</v>
       </c>
       <c r="L6">
         <f>((L4-L5)/L4)*100</f>
-        <v>75.823827539543657</v>
+        <v>9.9959583306200531E-3</v>
       </c>
       <c r="M6">
         <f>((M4-M5)/M4)*100</f>
-        <v>1.8275331902369348E-2</v>
+        <v>-9.001738508663662E-2</v>
       </c>
       <c r="O6">
         <f>((O4-O5)/O4)*100</f>
-        <v>98.794366694351481</v>
+        <v>-0.14855081909121434</v>
       </c>
       <c r="P6">
         <f>((P4-P5)/P4)*100</f>
-        <v>-1.53383657642925E-2</v>
+        <v>-0.20901290067759673</v>
       </c>
       <c r="R6">
         <f>((R4-R5)/R4)*100</f>
-        <v>98.323548909138765</v>
+        <v>6.352296115535074E-3</v>
       </c>
       <c r="S6">
         <f>((S4-S5)/S4)*100</f>
-        <v>-3.9150816714984731E-3</v>
+        <v>1.8181449220457616E-2</v>
       </c>
       <c r="U6">
         <f>((U4-U5)/U4)*100</f>
-        <v>96.983588313420526</v>
+        <v>2.3764077471449142E-3</v>
       </c>
       <c r="V6">
         <f>((V4-V5)/V4)*100</f>
-        <v>5.2696881875534066E-3</v>
+        <v>-2.1998297355475444E-2</v>
       </c>
       <c r="X6">
         <f>((X4-X5)/X4)*100</f>
-        <v>95.465851086659754</v>
+        <v>-7.8679267893968508E-2</v>
       </c>
       <c r="Y6">
         <f>((Y4-Y5)/Y4)*100</f>
-        <v>-6.6165150331572747E-2</v>
+        <v>-0.16767715743210254</v>
       </c>
       <c r="AA6">
         <f>((AA4-AA5)/AA4)*100</f>
-        <v>96.994229968320994</v>
+        <v>-2.7243396522026404E-2</v>
       </c>
       <c r="AB6">
         <f>((AB4-AB5)/AB4)*100</f>
-        <v>9.3652964459275539E-3</v>
+        <v>-6.4791881618371933E-2</v>
       </c>
       <c r="AD6">
         <f>((AD4-AD5)/AD4)*100</f>
-        <v>85.441885192023463</v>
+        <v>4.6259048672602429E-2</v>
       </c>
       <c r="AE6">
         <f>((AE4-AE5)/AE4)*100</f>
-        <v>-2.2412488665593273E-2</v>
+        <v>2.9691515750951521E-2</v>
       </c>
       <c r="AG6">
         <f>((AG4-AG5)/AG4)*100</f>
-        <v>99.590207870875858</v>
+        <v>-0.52987237927181707</v>
       </c>
       <c r="AH6">
         <f>((AH4-AH5)/AH4)*100</f>
-        <v>-4.0182434508662906E-2</v>
+        <v>-0.39387570034905117</v>
       </c>
       <c r="AJ6">
         <f>((AJ4-AJ5)/AJ4)*100</f>
-        <v>-1.9379795505074249</v>
+        <v>-0.30497054872574358</v>
       </c>
       <c r="AK6">
         <f>((AK4-AK5)/AK4)*100</f>
-        <v>0.62771900991408691</v>
+        <v>-1.0806723090527386</v>
       </c>
       <c r="AM6">
         <f>((AM4-AM5)/AM4)*100</f>
-        <v>85.659713516429363</v>
+        <v>-5.2874515339635716E-3</v>
       </c>
       <c r="AN6">
         <f>((AN4-AN5)/AN4)*100</f>
-        <v>5.3476771764439362E-3</v>
-      </c>
+        <v>-2.3864001774150271E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="B12" s="1"/>
+    </row>
+    <row r="13" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B14" s="1"/>
       <c r="T14" s="2"/>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1174,8 +1184,18 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:T2"/>
   </mergeCells>
+  <conditionalFormatting sqref="D6">
+    <cfRule type="colorScale" priority="60">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E4:E5">
-    <cfRule type="colorScale" priority="27">
+    <cfRule type="colorScale" priority="74">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1185,7 +1205,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H5">
-    <cfRule type="colorScale" priority="25">
+    <cfRule type="colorScale" priority="37">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1195,7 +1215,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:K5">
-    <cfRule type="colorScale" priority="24">
+    <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1205,7 +1225,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:N5">
-    <cfRule type="colorScale" priority="23">
+    <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1215,7 +1235,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q5">
-    <cfRule type="colorScale" priority="22">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1225,7 +1245,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T4:T5">
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1235,7 +1255,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W4:W5">
-    <cfRule type="colorScale" priority="20">
+    <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1245,7 +1265,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z4:Z5">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1255,7 +1275,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC4:AC5">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1265,7 +1285,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF4:AF5">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="29">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1275,7 +1295,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI4:AI5">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1285,7 +1305,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL4:AL5">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1295,7 +1315,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO4:AO5">
-    <cfRule type="colorScale" priority="14">
+    <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1304,132 +1324,252 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:D6">
-    <cfRule type="colorScale" priority="13">
+  <conditionalFormatting sqref="C6">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:G6">
-    <cfRule type="colorScale" priority="12">
+  <conditionalFormatting sqref="F6">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J6">
-    <cfRule type="colorScale" priority="11">
+  <conditionalFormatting sqref="G6">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:M6">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="I6">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6:P6">
-    <cfRule type="colorScale" priority="9">
+  <conditionalFormatting sqref="J6">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R6:S6">
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="L6">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U6:V6">
-    <cfRule type="colorScale" priority="7">
+  <conditionalFormatting sqref="M6">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X6:Y6">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="O6">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA6:AB6">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="P6">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD6:AE6">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="R6">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AG6:AH6">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="S6">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ6:AK6">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="U6">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM6:AN6">
+  <conditionalFormatting sqref="V6">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X6">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y6">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB6">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD6">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE6">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG6">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AH6">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ6">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK6">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM6">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN6">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFFF3500"/>
         <color rgb="FF92D050"/>
       </colorScale>
     </cfRule>
@@ -1443,7 +1583,7 @@
   <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" customWidth="1"/>
     <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
@@ -1539,43 +1679,43 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>4.7340293059999903</v>
+        <v>2.0945292000000001E-2</v>
       </c>
       <c r="D5">
-        <v>21.176729871999999</v>
+        <v>7.7977030729999903</v>
       </c>
       <c r="E5">
-        <v>9.4457361899999892</v>
+        <v>0.100677564</v>
       </c>
       <c r="F5">
-        <v>6.2217804140000004</v>
+        <v>1.51638297</v>
       </c>
       <c r="G5">
-        <v>4.7682641119999998</v>
+        <v>5.5917888000000103E-2</v>
       </c>
       <c r="H5">
-        <v>4.78634752199999</v>
+        <v>0.45915287100000002</v>
       </c>
       <c r="I5">
-        <v>4.8526370550000104</v>
+        <v>6.0677486629999997</v>
       </c>
       <c r="J5">
-        <v>4.9441060699999904</v>
+        <v>0.27247442699999902</v>
       </c>
       <c r="K5">
-        <v>4.8479211129999804</v>
+        <v>0.492297602</v>
       </c>
       <c r="L5">
-        <v>10.389432319999999</v>
+        <v>3.9035411389999899</v>
       </c>
       <c r="M5">
-        <v>4.73018520599999</v>
+        <v>1.9352582E-2</v>
       </c>
       <c r="N5">
-        <v>0.57304119499999995</v>
+        <v>0.61789860100000005</v>
       </c>
       <c r="O5">
-        <v>80.923910221</v>
+        <v>20.722267380000002</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -1583,43 +1723,43 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>4.7393095049999996</v>
+        <v>2.1359196999999899E-2</v>
       </c>
       <c r="D6">
-        <v>21.173363765999898</v>
+        <v>7.795109515</v>
       </c>
       <c r="E6">
-        <v>9.4572644579999796</v>
+        <v>0.10401200099999899</v>
       </c>
       <c r="F6">
-        <v>6.2261814449999999</v>
+        <v>1.5165825909999899</v>
       </c>
       <c r="G6">
-        <v>4.7731040329999903</v>
+        <v>5.6184010999999902E-2</v>
       </c>
       <c r="H6">
-        <v>4.7896122209999898</v>
+        <v>0.459507095999999</v>
       </c>
       <c r="I6">
-        <v>4.8602087559999996</v>
+        <v>6.063977951</v>
       </c>
       <c r="J6">
-        <v>4.9492782460000004</v>
+        <v>0.27396532500000098</v>
       </c>
       <c r="K6">
-        <v>4.8529851260000001</v>
+        <v>0.49250761799999898</v>
       </c>
       <c r="L6">
-        <v>10.393453508</v>
+        <v>3.9045517169999799</v>
       </c>
       <c r="M6">
-        <v>4.7350227470000004</v>
+        <v>1.967207E-2</v>
       </c>
       <c r="N6">
-        <v>0.57079999699999995</v>
+        <v>0.54323971000000004</v>
       </c>
       <c r="O6">
-        <v>80.976149698</v>
+        <v>20.724220821999999</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -1627,43 +1767,43 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>4.7078935550000001</v>
+        <v>2.0935884999999901E-2</v>
       </c>
       <c r="D7">
-        <v>21.146499433999999</v>
+        <v>7.7921811439999997</v>
       </c>
       <c r="E7">
-        <v>9.3944941359999898</v>
+        <v>0.101148921999999</v>
       </c>
       <c r="F7">
-        <v>6.1949537149999996</v>
+        <v>1.514309538</v>
       </c>
       <c r="G7">
-        <v>4.7398854799999999</v>
+        <v>5.585818E-2</v>
       </c>
       <c r="H7">
-        <v>4.7574510490000002</v>
+        <v>0.458939813999999</v>
       </c>
       <c r="I7">
-        <v>4.8284425640000102</v>
+        <v>6.0662435300000004</v>
       </c>
       <c r="J7">
-        <v>4.9171688830000102</v>
+        <v>0.27186163400000002</v>
       </c>
       <c r="K7">
-        <v>4.8211042189999898</v>
+        <v>0.491587261</v>
       </c>
       <c r="L7">
-        <v>10.363234916</v>
+        <v>3.90386092699999</v>
       </c>
       <c r="M7">
-        <v>4.7036561429999999</v>
+        <v>1.93052139999999E-2</v>
       </c>
       <c r="N7">
-        <v>0.57259144100000003</v>
+        <v>0.54461698599999997</v>
       </c>
       <c r="O7">
-        <v>80.601453527000004</v>
+        <v>20.712324318</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -1671,43 +1811,43 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>4.8357023659999996</v>
+        <v>2.08336719999999E-2</v>
       </c>
       <c r="D8">
-        <v>21.283297358999999</v>
+        <v>7.7812151570000001</v>
       </c>
       <c r="E8">
-        <v>9.6534851180000008</v>
+        <v>0.10033523599999999</v>
       </c>
       <c r="F8">
-        <v>6.3259116600000098</v>
+        <v>1.512441935</v>
       </c>
       <c r="G8">
-        <v>4.8699703429999897</v>
+        <v>5.5827926999999999E-2</v>
       </c>
       <c r="H8">
-        <v>4.8880030239999899</v>
+        <v>0.45860525600000002</v>
       </c>
       <c r="I8">
-        <v>4.9540698719999998</v>
+        <v>6.0625658989999902</v>
       </c>
       <c r="J8">
-        <v>5.0477363430000004</v>
+        <v>0.27135582499999999</v>
       </c>
       <c r="K8">
-        <v>4.9493739049999999</v>
+        <v>0.49157306899999997</v>
       </c>
       <c r="L8">
-        <v>10.490154618999901</v>
+        <v>3.9030260699999899</v>
       </c>
       <c r="M8">
-        <v>4.8317443500000001</v>
+        <v>1.9307754E-2</v>
       </c>
       <c r="N8">
-        <v>0.56438216600000002</v>
+        <v>0.54530207200000003</v>
       </c>
       <c r="O8">
-        <v>82.156601383999998</v>
+        <v>20.693376035</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -1715,43 +1855,43 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>4.7201029639999899</v>
+        <v>2.0906497E-2</v>
       </c>
       <c r="D9">
-        <v>21.162477132999999</v>
+        <v>7.7805381919999999</v>
       </c>
       <c r="E9">
-        <v>9.4234756789999992</v>
+        <v>0.100159464999999</v>
       </c>
       <c r="F9">
-        <v>6.2093324299999804</v>
+        <v>1.5116671129999899</v>
       </c>
       <c r="G9">
-        <v>4.7542486399999904</v>
+        <v>5.5745634000000002E-2</v>
       </c>
       <c r="H9">
-        <v>4.7723286930000004</v>
+        <v>0.45859409299999998</v>
       </c>
       <c r="I9">
-        <v>4.8406304889999996</v>
+        <v>6.0593861860000002</v>
       </c>
       <c r="J9">
-        <v>4.92910223999999</v>
+        <v>0.27132947599999901</v>
       </c>
       <c r="K9">
-        <v>4.8331939989999997</v>
+        <v>0.49138484900000001</v>
       </c>
       <c r="L9">
-        <v>10.376906498999899</v>
+        <v>3.9032113759999998</v>
       </c>
       <c r="M9">
-        <v>4.7158174270000002</v>
+        <v>1.9323584000000001E-2</v>
       </c>
       <c r="N9">
-        <v>0.57460502199999997</v>
+        <v>0.53678791199999998</v>
       </c>
       <c r="O9">
-        <v>80.764317835</v>
+        <v>20.688285358000002</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -1759,43 +1899,43 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>4.7483563999999898</v>
+        <v>2.08305289999999E-2</v>
       </c>
       <c r="D10">
-        <v>21.204867498999899</v>
+        <v>7.7814282109999997</v>
       </c>
       <c r="E10">
-        <v>9.4793780250000097</v>
+        <v>0.10019067299999999</v>
       </c>
       <c r="F10">
-        <v>6.2381119399999996</v>
+        <v>1.5114285030000001</v>
       </c>
       <c r="G10">
-        <v>4.7830271779999904</v>
+        <v>5.5645885000000103E-2</v>
       </c>
       <c r="H10">
-        <v>4.8021576899999898</v>
+        <v>0.45858836200000003</v>
       </c>
       <c r="I10">
-        <v>4.8694124350000001</v>
+        <v>6.0617983099999897</v>
       </c>
       <c r="J10">
-        <v>4.9590571159999897</v>
+        <v>0.27090224999999901</v>
       </c>
       <c r="K10">
-        <v>4.8623519149999801</v>
+        <v>0.49130033099999898</v>
       </c>
       <c r="L10">
-        <v>10.401261198</v>
+        <v>3.9017135810000001</v>
       </c>
       <c r="M10">
-        <v>4.74394939799999</v>
+        <v>1.9188847999999901E-2</v>
       </c>
       <c r="N10">
-        <v>0.55289784900000005</v>
+        <v>0.54013573299999995</v>
       </c>
       <c r="O10">
-        <v>81.118364749999998</v>
+        <v>20.689045309000001</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -1803,43 +1943,43 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>4.7037826629999904</v>
+        <v>2.1090906E-2</v>
       </c>
       <c r="D11">
-        <v>21.152131596</v>
+        <v>7.7843653549999896</v>
       </c>
       <c r="E11">
-        <v>9.3876109779999997</v>
+        <v>0.101818195</v>
       </c>
       <c r="F11">
-        <v>6.1921738199999998</v>
+        <v>1.512677534</v>
       </c>
       <c r="G11">
-        <v>4.73704256899999</v>
+        <v>5.5970686000000103E-2</v>
       </c>
       <c r="H11">
-        <v>4.7546049190000099</v>
+        <v>0.45885493099999902</v>
       </c>
       <c r="I11">
-        <v>4.8231421749999903</v>
+        <v>6.061748981</v>
       </c>
       <c r="J11">
-        <v>4.9121940719999904</v>
+        <v>0.272130135</v>
       </c>
       <c r="K11">
-        <v>4.8161531389999999</v>
+        <v>0.49171955099999898</v>
       </c>
       <c r="L11">
-        <v>10.356330882</v>
+        <v>3.8977867249999898</v>
       </c>
       <c r="M11">
-        <v>4.6991199909999901</v>
+        <v>1.9382218999999899E-2</v>
       </c>
       <c r="N11">
-        <v>0.55554261299999996</v>
+        <v>0.53911805499999998</v>
       </c>
       <c r="O11">
-        <v>80.560378224999994</v>
+        <v>20.693866938999999</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1847,43 +1987,43 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>4.6960157959999904</v>
+        <v>2.1049211999999901E-2</v>
       </c>
       <c r="D12">
-        <v>21.135143617000001</v>
+        <v>7.7794660599999803</v>
       </c>
       <c r="E12">
-        <v>9.3704731389999907</v>
+        <v>0.10056599300000001</v>
       </c>
       <c r="F12">
-        <v>6.1849777839999902</v>
+        <v>1.511711612</v>
       </c>
       <c r="G12">
-        <v>4.7298488310000097</v>
+        <v>5.5815807000000099E-2</v>
       </c>
       <c r="H12">
-        <v>4.74821225899999</v>
+        <v>0.45880408700000003</v>
       </c>
       <c r="I12">
-        <v>4.8161023499999898</v>
+        <v>6.0617813089999997</v>
       </c>
       <c r="J12">
-        <v>4.9041083179999996</v>
+        <v>0.27180590999999898</v>
       </c>
       <c r="K12">
-        <v>4.8065764169999996</v>
+        <v>0.49144501099999999</v>
       </c>
       <c r="L12">
-        <v>10.353393854</v>
+        <v>3.9043868549999901</v>
       </c>
       <c r="M12">
-        <v>4.6916778209999901</v>
+        <v>1.93601149999999E-2</v>
       </c>
       <c r="N12">
-        <v>0.55554574300000004</v>
+        <v>0.53863703100000004</v>
       </c>
       <c r="O12">
-        <v>80.462678502000003</v>
+        <v>20.692317829</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -1891,43 +2031,43 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>4.7152222879999997</v>
+        <v>2.1036944999999901E-2</v>
       </c>
       <c r="D13">
-        <v>21.163150134999899</v>
+        <v>7.7869990860000096</v>
       </c>
       <c r="E13">
-        <v>9.4112512409999898</v>
+        <v>0.100745107999999</v>
       </c>
       <c r="F13">
-        <v>6.2047871109999999</v>
+        <v>1.513208957</v>
       </c>
       <c r="G13">
-        <v>4.7493141909999999</v>
+        <v>5.5890241000000097E-2</v>
       </c>
       <c r="H13">
-        <v>4.7671523330000003</v>
+        <v>0.45893628199999997</v>
       </c>
       <c r="I13">
-        <v>4.8345936519999997</v>
+        <v>6.0607884379999897</v>
       </c>
       <c r="J13">
-        <v>4.9243923099999902</v>
+        <v>0.27208739399999998</v>
       </c>
       <c r="K13">
-        <v>4.8269851900000003</v>
+        <v>0.491826123</v>
       </c>
       <c r="L13">
-        <v>10.369362314</v>
+        <v>3.8965046640000001</v>
       </c>
       <c r="M13">
-        <v>4.7109683779999898</v>
+        <v>1.9376067999999899E-2</v>
       </c>
       <c r="N13">
-        <v>0.56577272000000001</v>
+        <v>0.54174849199999997</v>
       </c>
       <c r="O13">
-        <v>80.705057595</v>
+        <v>20.693725327999999</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -1935,43 +2075,43 @@
         <v>9</v>
       </c>
       <c r="C14">
-        <v>4.7611054549999903</v>
+        <v>2.1146714E-2</v>
       </c>
       <c r="D14">
-        <v>21.208750736999999</v>
+        <v>7.7893656160000004</v>
       </c>
       <c r="E14">
-        <v>9.4983145119999808</v>
+        <v>0.10103263</v>
       </c>
       <c r="F14">
-        <v>6.2516233699999999</v>
+        <v>1.5128756209999901</v>
       </c>
       <c r="G14">
-        <v>4.7949720709999903</v>
+        <v>5.5926254000000002E-2</v>
       </c>
       <c r="H14">
-        <v>4.8131857169999996</v>
+        <v>0.45909798600000001</v>
       </c>
       <c r="I14">
-        <v>4.8818332839999803</v>
+        <v>6.0629500860000096</v>
       </c>
       <c r="J14">
-        <v>4.9705023209999997</v>
+        <v>0.27244211800000001</v>
       </c>
       <c r="K14">
-        <v>4.8743232359999897</v>
+        <v>0.49190621499999898</v>
       </c>
       <c r="L14">
-        <v>10.414609773</v>
+        <v>3.89601520899999</v>
       </c>
       <c r="M14">
-        <v>4.7569945640000002</v>
+        <v>1.9431583999999901E-2</v>
       </c>
       <c r="N14">
-        <v>0.55453468500000003</v>
+        <v>0.54003348799999995</v>
       </c>
       <c r="O14">
-        <v>81.252443843999998</v>
+        <v>20.698236467000001</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -1979,43 +2119,43 @@
         <v>21</v>
       </c>
       <c r="C15" s="1">
-        <v>4.7361520297999897</v>
+        <v>2.10134848999999E-2</v>
       </c>
       <c r="D15" s="1">
-        <v>21.1806411148</v>
+        <v>7.7868371409000003</v>
       </c>
       <c r="E15" s="1">
-        <v>9.4521483475999908</v>
+        <v>0.10106857869999999</v>
       </c>
       <c r="F15" s="1">
-        <v>6.2249833689000003</v>
+        <v>1.5133286373999999</v>
       </c>
       <c r="G15" s="1">
-        <v>4.7699677447999997</v>
+        <v>5.5878251300000001E-2</v>
       </c>
       <c r="H15" s="1">
-        <v>4.7879055426999999</v>
+        <v>0.45890807779999998</v>
       </c>
       <c r="I15" s="1">
-        <v>4.8561072632000002</v>
+        <v>6.0628989352999998</v>
       </c>
       <c r="J15" s="1">
-        <v>4.9457645918999997</v>
+        <v>0.27203544940000002</v>
       </c>
       <c r="K15" s="1">
-        <v>4.8490968258999896</v>
+        <v>0.49175476299999998</v>
       </c>
       <c r="L15" s="1">
-        <v>10.3908139883</v>
+        <v>3.9014598262999902</v>
       </c>
       <c r="M15" s="1">
-        <v>4.7319136024999997</v>
+        <v>1.93700037999999E-2</v>
       </c>
       <c r="N15" s="1">
-        <v>0.56397134309999997</v>
+        <v>0.54875180800000001</v>
       </c>
       <c r="O15" s="1">
-        <v>80.952135558099997</v>
+        <v>20.700766578500001</v>
       </c>
     </row>
   </sheetData>
@@ -2113,43 +2253,43 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>2.1720421999999899E-2</v>
+        <v>2.1101384000000001E-2</v>
       </c>
       <c r="D5">
-        <v>7.7920159560000002</v>
+        <v>7.79302745099998</v>
       </c>
       <c r="E5">
-        <v>9.8926041000000201E-2</v>
+        <v>0.100698307</v>
       </c>
       <c r="F5">
-        <v>1.514987834</v>
+        <v>1.5172041649999899</v>
       </c>
       <c r="G5">
-        <v>5.6670711999999998E-2</v>
+        <v>5.5791908000000001E-2</v>
       </c>
       <c r="H5">
-        <v>0.45792223899999901</v>
+        <v>0.45921943500000001</v>
       </c>
       <c r="I5">
-        <v>6.0629683709999904</v>
+        <v>6.0636783699999901</v>
       </c>
       <c r="J5">
-        <v>0.27254366399999902</v>
+        <v>0.27255087899999902</v>
       </c>
       <c r="K5">
-        <v>0.492584572</v>
+        <v>0.49235883599999802</v>
       </c>
       <c r="L5">
-        <v>3.9054659680000001</v>
+        <v>3.9059577489999899</v>
       </c>
       <c r="M5">
-        <v>2.0203208E-2</v>
+        <v>1.94064139999999E-2</v>
       </c>
       <c r="N5">
-        <v>0.64593537300000003</v>
+        <v>0.61528601199999999</v>
       </c>
       <c r="O5">
-        <v>20.713234384</v>
+        <v>20.717549983000001</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2157,43 +2297,43 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>2.1932872999999901E-2</v>
+        <v>2.1279628999999901E-2</v>
       </c>
       <c r="D6">
-        <v>7.7932568639999804</v>
+        <v>7.79709311199999</v>
       </c>
       <c r="E6">
-        <v>0.100150211999999</v>
+        <v>0.101755966</v>
       </c>
       <c r="F6">
-        <v>1.5148518119999901</v>
+        <v>1.5162854719999901</v>
       </c>
       <c r="G6">
-        <v>5.6832657999999897E-2</v>
+        <v>5.60827320000001E-2</v>
       </c>
       <c r="H6">
-        <v>0.45801357599999998</v>
+        <v>0.45925363499999999</v>
       </c>
       <c r="I6">
-        <v>6.0620578969999999</v>
+        <v>6.0638862659999901</v>
       </c>
       <c r="J6">
-        <v>0.27391537499999902</v>
+        <v>0.27413057499999899</v>
       </c>
       <c r="K6">
-        <v>0.49292541600000001</v>
+        <v>0.492675635</v>
       </c>
       <c r="L6">
-        <v>3.8996984129999999</v>
+        <v>3.9011064999999898</v>
       </c>
       <c r="M6">
-        <v>2.0393437E-2</v>
+        <v>1.9632154999999998E-2</v>
       </c>
       <c r="N6">
-        <v>0.550244972</v>
+        <v>0.54432430300000001</v>
       </c>
       <c r="O6">
-        <v>20.712029911999998</v>
+        <v>20.719638375999999</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -2201,43 +2341,43 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>2.1673924000000001E-2</v>
+        <v>2.0974719999999902E-2</v>
       </c>
       <c r="D7">
-        <v>7.78517397500001</v>
+        <v>7.7970552969999902</v>
       </c>
       <c r="E7">
-        <v>9.8263606000000295E-2</v>
+        <v>0.101015059</v>
       </c>
       <c r="F7">
-        <v>1.5145982249999901</v>
+        <v>1.51517175599999</v>
       </c>
       <c r="G7">
-        <v>5.6453717E-2</v>
+        <v>5.5776628000000002E-2</v>
       </c>
       <c r="H7">
-        <v>0.45786797299999998</v>
+        <v>0.45908050299999897</v>
       </c>
       <c r="I7">
-        <v>6.06432882399998</v>
+        <v>6.0662717739999996</v>
       </c>
       <c r="J7">
-        <v>0.272134289999999</v>
+        <v>0.27210804100000002</v>
       </c>
       <c r="K7">
-        <v>0.49234655300000002</v>
+        <v>0.49236375399999999</v>
       </c>
       <c r="L7">
-        <v>3.9066906959999899</v>
+        <v>3.9055599729999999</v>
       </c>
       <c r="M7">
-        <v>2.0032529E-2</v>
+        <v>1.93282919999999E-2</v>
       </c>
       <c r="N7">
-        <v>0.57788008999999996</v>
+        <v>0.54036128100000003</v>
       </c>
       <c r="O7">
-        <v>20.706679097999999</v>
+        <v>20.720896796000002</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -2245,43 +2385,43 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>2.1524842999999998E-2</v>
+        <v>2.0956139999999901E-2</v>
       </c>
       <c r="D8">
-        <v>7.7903554359999898</v>
+        <v>7.7877697669999897</v>
       </c>
       <c r="E8">
-        <v>9.8635195999999897E-2</v>
+        <v>9.9885357999999896E-2</v>
       </c>
       <c r="F8">
-        <v>1.51497759599999</v>
+        <v>1.51211037499999</v>
       </c>
       <c r="G8">
-        <v>5.6425546999999902E-2</v>
+        <v>5.5762935999999999E-2</v>
       </c>
       <c r="H8">
-        <v>0.45780708199999898</v>
+        <v>0.45854220199999901</v>
       </c>
       <c r="I8">
-        <v>6.06703356199999</v>
+        <v>6.0622401990000103</v>
       </c>
       <c r="J8">
-        <v>0.27221806099999901</v>
+        <v>0.27117142399999999</v>
       </c>
       <c r="K8">
-        <v>0.49258481599999798</v>
+        <v>0.491552883</v>
       </c>
       <c r="L8">
-        <v>3.90604397499999</v>
+        <v>3.8963203659999901</v>
       </c>
       <c r="M8">
-        <v>2.0019353999999899E-2</v>
+        <v>1.9265055E-2</v>
       </c>
       <c r="N8">
-        <v>0.54926370899999999</v>
+        <v>0.550553124</v>
       </c>
       <c r="O8">
-        <v>20.714700707999999</v>
+        <v>20.691628844</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2289,43 +2429,43 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>2.1505045999999899E-2</v>
+        <v>2.0884650000000001E-2</v>
       </c>
       <c r="D9">
-        <v>7.79237521900001</v>
+        <v>7.7794520330000099</v>
       </c>
       <c r="E9">
-        <v>9.8110879999999998E-2</v>
+        <v>0.10029113200000001</v>
       </c>
       <c r="F9">
-        <v>1.514759403</v>
+        <v>1.5121290780000001</v>
       </c>
       <c r="G9">
-        <v>5.6454982000000001E-2</v>
+        <v>5.5753456999999999E-2</v>
       </c>
       <c r="H9">
-        <v>0.45782401499999897</v>
+        <v>0.45871501999999897</v>
       </c>
       <c r="I9">
-        <v>6.0658227059999996</v>
+        <v>6.0606006370000101</v>
       </c>
       <c r="J9">
-        <v>0.27235633199999898</v>
+        <v>0.27122294399999902</v>
       </c>
       <c r="K9">
-        <v>0.492267179</v>
+        <v>0.49128346099999998</v>
       </c>
       <c r="L9">
-        <v>3.9025007180000002</v>
+        <v>3.9011952289999901</v>
       </c>
       <c r="M9">
-        <v>2.0040321E-2</v>
+        <v>1.9221643999999899E-2</v>
       </c>
       <c r="N9">
-        <v>0.54740489599999997</v>
+        <v>0.54035476100000002</v>
       </c>
       <c r="O9">
-        <v>20.711233804999999</v>
+        <v>20.686977975000001</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -2333,43 +2473,43 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>2.1446732999999999E-2</v>
+        <v>2.0807343999999901E-2</v>
       </c>
       <c r="D10">
-        <v>7.79217742799998</v>
+        <v>7.7878391180000097</v>
       </c>
       <c r="E10">
-        <v>9.8305396999999906E-2</v>
+        <v>9.9926715000000096E-2</v>
       </c>
       <c r="F10">
-        <v>1.51437720799999</v>
+        <v>1.5117757669999901</v>
       </c>
       <c r="G10">
-        <v>5.6399120000000101E-2</v>
+        <v>5.5649369999999997E-2</v>
       </c>
       <c r="H10">
-        <v>0.45764157999999899</v>
+        <v>0.45859571700000001</v>
       </c>
       <c r="I10">
-        <v>6.0663063140000002</v>
+        <v>6.0603357109999996</v>
       </c>
       <c r="J10">
-        <v>0.27173915100000001</v>
+        <v>0.27112144100000002</v>
       </c>
       <c r="K10">
-        <v>0.49202296899999898</v>
+        <v>0.49142884599999898</v>
       </c>
       <c r="L10">
-        <v>3.9073114050000002</v>
+        <v>3.9000256759999998</v>
       </c>
       <c r="M10">
-        <v>1.9971797999999999E-2</v>
+        <v>1.9312329999999999E-2</v>
       </c>
       <c r="N10">
-        <v>0.54614090900000001</v>
+        <v>0.53915951100000004</v>
       </c>
       <c r="O10">
-        <v>20.714789747000001</v>
+        <v>20.692864118999999</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2377,43 +2517,43 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>2.1616896999999899E-2</v>
+        <v>2.1106718999999899E-2</v>
       </c>
       <c r="D11">
-        <v>7.7921428089999898</v>
+        <v>7.7843844669999802</v>
       </c>
       <c r="E11">
-        <v>9.9132750000000006E-2</v>
+        <v>0.100622691</v>
       </c>
       <c r="F11">
-        <v>1.5150120439999899</v>
+        <v>1.51220974199999</v>
       </c>
       <c r="G11">
-        <v>5.6688913E-2</v>
+        <v>5.5990173999999997E-2</v>
       </c>
       <c r="H11">
-        <v>0.45803382599999998</v>
+        <v>0.458783633999999</v>
       </c>
       <c r="I11">
-        <v>6.0665790959999804</v>
+        <v>6.0625688519999903</v>
       </c>
       <c r="J11">
-        <v>0.27280712099999999</v>
+        <v>0.271670675999999</v>
       </c>
       <c r="K11">
-        <v>0.49276028799999899</v>
+        <v>0.49157911700000001</v>
       </c>
       <c r="L11">
-        <v>3.9066536109999901</v>
+        <v>3.89965502799999</v>
       </c>
       <c r="M11">
-        <v>2.0168087000000001E-2</v>
+        <v>1.9355522999999899E-2</v>
       </c>
       <c r="N11">
-        <v>0.54705949499999995</v>
+        <v>0.53928374499999998</v>
       </c>
       <c r="O11">
-        <v>20.718696206000001</v>
+        <v>20.694036471</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -2421,43 +2561,43 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>2.1699502999999998E-2</v>
+        <v>2.1055265999999899E-2</v>
       </c>
       <c r="D12">
-        <v>7.7960570239999702</v>
+        <v>7.7870121919999997</v>
       </c>
       <c r="E12">
-        <v>9.8950826000000006E-2</v>
+        <v>0.10130739499999999</v>
       </c>
       <c r="F12">
-        <v>1.5138778100000001</v>
+        <v>1.51215378999999</v>
       </c>
       <c r="G12">
-        <v>5.6606003000000002E-2</v>
+        <v>5.5870721999999901E-2</v>
       </c>
       <c r="H12">
-        <v>0.45791276199999997</v>
+        <v>0.45870782199999999</v>
       </c>
       <c r="I12">
-        <v>6.0653505989999896</v>
+        <v>6.0600565519999998</v>
       </c>
       <c r="J12">
-        <v>0.27221119799999999</v>
+        <v>0.272015848</v>
       </c>
       <c r="K12">
-        <v>0.49230500999999999</v>
+        <v>0.491494870999999</v>
       </c>
       <c r="L12">
-        <v>3.9038788939999902</v>
+        <v>3.902312512</v>
       </c>
       <c r="M12">
-        <v>2.0186594999999901E-2</v>
+        <v>1.9278192999999999E-2</v>
       </c>
       <c r="N12">
-        <v>0.54342701900000001</v>
+        <v>0.53867469499999998</v>
       </c>
       <c r="O12">
-        <v>20.716681764</v>
+        <v>20.697453193000001</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -2465,43 +2605,43 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>2.17129459999999E-2</v>
+        <v>2.1009811999999999E-2</v>
       </c>
       <c r="D13">
-        <v>7.78897069599999</v>
+        <v>7.78079164399999</v>
       </c>
       <c r="E13">
-        <v>9.8518339000000094E-2</v>
+        <v>0.101113538999999</v>
       </c>
       <c r="F13">
-        <v>1.51190811199999</v>
+        <v>1.5124974799999999</v>
       </c>
       <c r="G13">
-        <v>5.6603623999999998E-2</v>
+        <v>5.5813125999999998E-2</v>
       </c>
       <c r="H13">
-        <v>0.45760492600000002</v>
+        <v>0.45869143800000001</v>
       </c>
       <c r="I13">
-        <v>6.0605655199999902</v>
+        <v>6.0603539730000104</v>
       </c>
       <c r="J13">
-        <v>0.27217079099999902</v>
+        <v>0.27183335199999897</v>
       </c>
       <c r="K13">
-        <v>0.49201673399999901</v>
+        <v>0.491635667</v>
       </c>
       <c r="L13">
-        <v>3.8966925989999899</v>
+        <v>3.900215749</v>
       </c>
       <c r="M13">
-        <v>2.0140801E-2</v>
+        <v>1.9421697000000002E-2</v>
       </c>
       <c r="N13">
-        <v>0.54602609599999996</v>
+        <v>0.53861486400000003</v>
       </c>
       <c r="O13">
-        <v>20.694066958000001</v>
+        <v>20.689566696</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -2509,43 +2649,43 @@
         <v>9</v>
       </c>
       <c r="C14">
-        <v>2.1838885999999901E-2</v>
+        <v>2.1267149999999999E-2</v>
       </c>
       <c r="D14">
-        <v>7.7851553749999898</v>
+        <v>7.78856586200002</v>
       </c>
       <c r="E14">
-        <v>9.9621060999999997E-2</v>
+        <v>0.101402716</v>
       </c>
       <c r="F14">
-        <v>1.5120986300000001</v>
+        <v>1.5126722690000001</v>
       </c>
       <c r="G14">
-        <v>5.6726833000000101E-2</v>
+        <v>5.60558099999999E-2</v>
       </c>
       <c r="H14">
-        <v>0.458101534999999</v>
+        <v>0.45901620999999998</v>
       </c>
       <c r="I14">
-        <v>6.0625183060000003</v>
+        <v>6.0629085410000103</v>
       </c>
       <c r="J14">
-        <v>0.272697946999999</v>
+        <v>0.272708176999999</v>
       </c>
       <c r="K14">
-        <v>0.49205622700000001</v>
+        <v>0.49192058099999902</v>
       </c>
       <c r="L14">
-        <v>3.9075642240000001</v>
+        <v>3.8957304859999899</v>
       </c>
       <c r="M14">
-        <v>2.0250283000000001E-2</v>
+        <v>1.9526368999999998E-2</v>
       </c>
       <c r="N14">
-        <v>0.54671930899999999</v>
+        <v>0.54182851099999996</v>
       </c>
       <c r="O14">
-        <v>20.705938906</v>
+        <v>20.698456970999999</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -2553,43 +2693,43 @@
         <v>22</v>
       </c>
       <c r="C15" s="1">
-        <v>2.1667207299999901E-2</v>
+        <v>2.1044281399999899E-2</v>
       </c>
       <c r="D15" s="1">
-        <v>7.7907680781999904</v>
+        <v>7.7882990942999903</v>
       </c>
       <c r="E15" s="1">
-        <v>9.8861430799999997E-2</v>
+        <v>0.1008018878</v>
       </c>
       <c r="F15" s="1">
-        <v>1.51414486739999</v>
+        <v>1.5134209893999899</v>
       </c>
       <c r="G15" s="1">
-        <v>5.6586210900000003E-2</v>
+        <v>5.5854686299999998E-2</v>
       </c>
       <c r="H15" s="1">
-        <v>0.45787295140000001</v>
+        <v>0.45886056159999999</v>
       </c>
       <c r="I15" s="1">
-        <v>6.06435311949999</v>
+        <v>6.0622900875000001</v>
       </c>
       <c r="J15" s="1">
-        <v>0.27247939299999901</v>
+        <v>0.27205333569999901</v>
       </c>
       <c r="K15" s="1">
-        <v>0.49238697640000001</v>
+        <v>0.49182936509999903</v>
       </c>
       <c r="L15" s="1">
-        <v>3.9042500502999902</v>
+        <v>3.9008079268000002</v>
       </c>
       <c r="M15" s="1">
-        <v>2.0140641300000001E-2</v>
+        <v>1.93747672E-2</v>
       </c>
       <c r="N15" s="1">
-        <v>0.56001018679999903</v>
+        <v>0.54884408070000001</v>
       </c>
       <c r="O15" s="1">
-        <v>20.710805148799999</v>
+        <v>20.7009069424</v>
       </c>
     </row>
   </sheetData>
@@ -2687,43 +2827,43 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>2.0424912999999999E-2</v>
+        <v>2.1066069999999999E-2</v>
       </c>
       <c r="D5">
-        <v>7.7867697349999903</v>
+        <v>7.7994737460000003</v>
       </c>
       <c r="E5">
-        <v>9.1322597999999894E-2</v>
+        <v>0.101644125</v>
       </c>
       <c r="F5">
-        <v>1.5043494099999899</v>
+        <v>1.5162155929999901</v>
       </c>
       <c r="G5">
-        <v>5.7297887999999901E-2</v>
+        <v>5.5874482000000003E-2</v>
       </c>
       <c r="H5">
-        <v>8.0126062999999803E-2</v>
+        <v>0.45912639099999902</v>
       </c>
       <c r="I5">
-        <v>0.14635807000000001</v>
+        <v>6.0657522789999998</v>
       </c>
       <c r="J5">
-        <v>0.22410363699999999</v>
+        <v>0.27239945999999998</v>
       </c>
       <c r="K5">
-        <v>0.145887511</v>
+        <v>0.49202833999999901</v>
       </c>
       <c r="L5">
-        <v>1.5135437140000001</v>
+        <v>3.9017833849999999</v>
       </c>
       <c r="M5">
-        <v>1.9270493999999899E-2</v>
+        <v>1.9374984000000001E-2</v>
       </c>
       <c r="N5">
-        <v>0.63718657899999998</v>
+        <v>0.616310998</v>
       </c>
       <c r="O5">
-        <v>11.605081670000001</v>
+        <v>20.72091713</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2731,43 +2871,43 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>2.1145951E-2</v>
+        <v>2.2013108999999999E-2</v>
       </c>
       <c r="D6">
-        <v>7.7860681689999902</v>
+        <v>7.8010432889999999</v>
       </c>
       <c r="E6">
-        <v>9.1019702999999993E-2</v>
+        <v>0.101714957999999</v>
       </c>
       <c r="F6">
-        <v>1.504760248</v>
+        <v>1.51559118599999</v>
       </c>
       <c r="G6">
-        <v>5.8056615999999998E-2</v>
+        <v>5.6949554999999999E-2</v>
       </c>
       <c r="H6">
-        <v>7.9142330999999899E-2</v>
+        <v>0.45848459899999999</v>
       </c>
       <c r="I6">
-        <v>0.14721379100000001</v>
+        <v>6.0653772449999996</v>
       </c>
       <c r="J6">
-        <v>0.22464350599999999</v>
+        <v>0.27441423099999901</v>
       </c>
       <c r="K6">
-        <v>0.14654013999999899</v>
+        <v>0.493028518999999</v>
       </c>
       <c r="L6">
-        <v>1.5158264749999999</v>
+        <v>3.8995791579999901</v>
       </c>
       <c r="M6">
-        <v>2.0120513999999999E-2</v>
+        <v>2.0546848E-2</v>
       </c>
       <c r="N6">
-        <v>0.58061084600000001</v>
+        <v>0.55257705899999998</v>
       </c>
       <c r="O6">
-        <v>11.611603560000001</v>
+        <v>20.726886456999999</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -2775,43 +2915,43 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>2.0321663E-2</v>
+        <v>2.1102395999999898E-2</v>
       </c>
       <c r="D7">
-        <v>7.7858370370000003</v>
+        <v>7.7918346869999997</v>
       </c>
       <c r="E7">
-        <v>9.1435814000000198E-2</v>
+        <v>0.101059461</v>
       </c>
       <c r="F7">
-        <v>1.50463510299999</v>
+        <v>1.513774784</v>
       </c>
       <c r="G7">
-        <v>5.7139267999999903E-2</v>
+        <v>5.5743058999999998E-2</v>
       </c>
       <c r="H7">
-        <v>8.0468895999999998E-2</v>
+        <v>0.45918726999999998</v>
       </c>
       <c r="I7">
-        <v>0.146477828</v>
+        <v>6.0655896979999904</v>
       </c>
       <c r="J7">
-        <v>0.22378975800000001</v>
+        <v>0.27184363299999997</v>
       </c>
       <c r="K7">
-        <v>0.14580547599999999</v>
+        <v>0.49198598100000002</v>
       </c>
       <c r="L7">
-        <v>1.5118537869999999</v>
+        <v>3.9020698170000001</v>
       </c>
       <c r="M7">
-        <v>1.9273346999999899E-2</v>
+        <v>1.9253632999999899E-2</v>
       </c>
       <c r="N7">
-        <v>0.56270112800000005</v>
+        <v>0.54308842300000004</v>
       </c>
       <c r="O7">
-        <v>11.603158564999999</v>
+        <v>20.709690736999999</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -2819,43 +2959,43 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>2.0864639000000001E-2</v>
+        <v>2.0968386999999901E-2</v>
       </c>
       <c r="D8">
-        <v>7.791942186</v>
+        <v>7.7860453190000101</v>
       </c>
       <c r="E8">
-        <v>9.3432404999999899E-2</v>
+        <v>0.100349826</v>
       </c>
       <c r="F8">
-        <v>1.5056955270000001</v>
+        <v>1.512698646</v>
       </c>
       <c r="G8">
-        <v>5.7837718999999899E-2</v>
+        <v>5.5743950000000098E-2</v>
       </c>
       <c r="H8">
-        <v>8.0883411999999794E-2</v>
+        <v>0.45916385300000001</v>
       </c>
       <c r="I8">
-        <v>0.14729577499999999</v>
+        <v>6.0618285339999902</v>
       </c>
       <c r="J8">
-        <v>0.22659679099999999</v>
+        <v>0.27276218800000002</v>
       </c>
       <c r="K8">
-        <v>0.14671094299999901</v>
+        <v>0.49155756699999997</v>
       </c>
       <c r="L8">
-        <v>1.5164940629999999</v>
+        <v>3.8938646370000001</v>
       </c>
       <c r="M8">
-        <v>1.9708712999999999E-2</v>
+        <v>1.9304002000000001E-2</v>
       </c>
       <c r="N8">
-        <v>0.56443909199999998</v>
+        <v>0.54494798700000002</v>
       </c>
       <c r="O8">
-        <v>11.62344429</v>
+        <v>20.690456955999998</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -2863,43 +3003,43 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>2.0280942999999899E-2</v>
+        <v>2.0973215999999899E-2</v>
       </c>
       <c r="D9">
-        <v>7.7999430569999904</v>
+        <v>7.7813027589999901</v>
       </c>
       <c r="E9">
-        <v>9.0877374999999802E-2</v>
+        <v>0.101126643</v>
       </c>
       <c r="F9">
-        <v>1.50655010599999</v>
+        <v>1.5121788599999899</v>
       </c>
       <c r="G9">
-        <v>5.7248313999999897E-2</v>
+        <v>5.5740315999999998E-2</v>
       </c>
       <c r="H9">
-        <v>8.0485838000000101E-2</v>
+        <v>0.45859746899999898</v>
       </c>
       <c r="I9">
-        <v>0.14656117699999999</v>
+        <v>6.0613853170000001</v>
       </c>
       <c r="J9">
-        <v>0.22409077799999999</v>
+        <v>0.27138312999999897</v>
       </c>
       <c r="K9">
-        <v>0.14573356700000001</v>
+        <v>0.49132802600000097</v>
       </c>
       <c r="L9">
-        <v>1.51249728199999</v>
+        <v>3.9025352089999998</v>
       </c>
       <c r="M9">
-        <v>1.9202230000000001E-2</v>
+        <v>1.9322946999999899E-2</v>
       </c>
       <c r="N9">
-        <v>0.562185775</v>
+        <v>0.53796646000000004</v>
       </c>
       <c r="O9">
-        <v>11.619479439999999</v>
+        <v>20.692053219000002</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -2907,43 +3047,43 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>2.043876E-2</v>
+        <v>2.095733E-2</v>
       </c>
       <c r="D10">
-        <v>7.7974293039999996</v>
+        <v>7.7859232969999903</v>
       </c>
       <c r="E10">
-        <v>9.1080436999999903E-2</v>
+        <v>0.101294805</v>
       </c>
       <c r="F10">
-        <v>1.5064454389999899</v>
+        <v>1.51144327999999</v>
       </c>
       <c r="G10">
-        <v>5.7185278999999797E-2</v>
+        <v>5.5792281000000103E-2</v>
       </c>
       <c r="H10">
-        <v>8.0402278999999993E-2</v>
+        <v>0.45866275299999898</v>
       </c>
       <c r="I10">
-        <v>0.14645081199999899</v>
+        <v>6.0614671599999896</v>
       </c>
       <c r="J10">
-        <v>0.22453524499999999</v>
+        <v>0.27114375799999901</v>
       </c>
       <c r="K10">
-        <v>0.145886615999999</v>
+        <v>0.491510909</v>
       </c>
       <c r="L10">
-        <v>1.511602659</v>
+        <v>3.9005954509999898</v>
       </c>
       <c r="M10">
-        <v>1.9318756999999999E-2</v>
+        <v>1.9233350999999999E-2</v>
       </c>
       <c r="N10">
-        <v>0.57984765400000005</v>
+        <v>0.54721948499999995</v>
       </c>
       <c r="O10">
-        <v>11.616513956</v>
+        <v>20.694206857000001</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2951,43 +3091,43 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>2.0353184E-2</v>
+        <v>2.10826109999999E-2</v>
       </c>
       <c r="D11">
-        <v>7.7924300309999897</v>
+        <v>7.7838895780000099</v>
       </c>
       <c r="E11">
-        <v>9.0809097000000102E-2</v>
+        <v>0.10192346100000001</v>
       </c>
       <c r="F11">
-        <v>1.5053146959999999</v>
+        <v>1.512189867</v>
       </c>
       <c r="G11">
-        <v>5.7189707999999902E-2</v>
+        <v>5.5874761000000002E-2</v>
       </c>
       <c r="H11">
-        <v>8.0279349E-2</v>
+        <v>0.45884820900000001</v>
       </c>
       <c r="I11">
-        <v>0.146382653999999</v>
+        <v>6.0617735640000001</v>
       </c>
       <c r="J11">
-        <v>0.22355650699999999</v>
+        <v>0.271952155999999</v>
       </c>
       <c r="K11">
-        <v>0.14538958199999999</v>
+        <v>0.49183482699999898</v>
       </c>
       <c r="L11">
-        <v>1.513626312</v>
+        <v>3.8974218359999999</v>
       </c>
       <c r="M11">
-        <v>1.9171847999999901E-2</v>
+        <v>1.9351515E-2</v>
       </c>
       <c r="N11">
-        <v>0.560336846</v>
+        <v>0.53907629400000001</v>
       </c>
       <c r="O11">
-        <v>11.610014887</v>
+        <v>20.692990059</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -2995,43 +3135,43 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>2.0289628999999899E-2</v>
+        <v>2.1112009000000001E-2</v>
       </c>
       <c r="D12">
-        <v>7.7860702429999904</v>
+        <v>7.7827500570000003</v>
       </c>
       <c r="E12">
-        <v>9.1088189E-2</v>
+        <v>0.101276436</v>
       </c>
       <c r="F12">
-        <v>1.5032416559999899</v>
+        <v>1.511931492</v>
       </c>
       <c r="G12">
-        <v>5.7050234999999901E-2</v>
+        <v>5.5863916999999999E-2</v>
       </c>
       <c r="H12">
-        <v>8.02704679999999E-2</v>
+        <v>0.45887003999999998</v>
       </c>
       <c r="I12">
-        <v>0.14590045199999899</v>
+        <v>6.0604057690000097</v>
       </c>
       <c r="J12">
-        <v>0.223113902999999</v>
+        <v>0.27196870099999998</v>
       </c>
       <c r="K12">
-        <v>0.14498377500000001</v>
+        <v>0.491854862</v>
       </c>
       <c r="L12">
-        <v>1.51002137499999</v>
+        <v>3.9037895489999901</v>
       </c>
       <c r="M12">
-        <v>1.9153499000000001E-2</v>
+        <v>1.9461340000000001E-2</v>
       </c>
       <c r="N12">
-        <v>0.56179270699999995</v>
+        <v>0.54147638300000001</v>
       </c>
       <c r="O12">
-        <v>11.596820626</v>
+        <v>20.695688261000001</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -3039,43 +3179,43 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>2.03218539999999E-2</v>
+        <v>2.1062636999999901E-2</v>
       </c>
       <c r="D13">
-        <v>7.7836237120000096</v>
+        <v>7.7881428579999898</v>
       </c>
       <c r="E13">
-        <v>9.1111495999999903E-2</v>
+        <v>0.10146572199999999</v>
       </c>
       <c r="F13">
-        <v>1.5051262249999999</v>
+        <v>1.5128203149999899</v>
       </c>
       <c r="G13">
-        <v>5.7253967999999898E-2</v>
+        <v>5.5973003999999903E-2</v>
       </c>
       <c r="H13">
-        <v>8.0286094000000099E-2</v>
+        <v>0.45890385499999897</v>
       </c>
       <c r="I13">
-        <v>0.145972402</v>
+        <v>6.0601249340000001</v>
       </c>
       <c r="J13">
-        <v>0.22355931900000001</v>
+        <v>0.27200566399999998</v>
       </c>
       <c r="K13">
-        <v>0.145110973999999</v>
+        <v>0.49187511699999997</v>
       </c>
       <c r="L13">
-        <v>1.511406241</v>
+        <v>3.89971205599999</v>
       </c>
       <c r="M13">
-        <v>1.9221361999999999E-2</v>
+        <v>1.9399731E-2</v>
       </c>
       <c r="N13">
-        <v>0.58119497399999998</v>
+        <v>0.53865003</v>
       </c>
       <c r="O13">
-        <v>11.598596659</v>
+        <v>20.697728300000001</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -3083,43 +3223,43 @@
         <v>9</v>
       </c>
       <c r="C14">
-        <v>2.04681699999999E-2</v>
+        <v>2.1142463E-2</v>
       </c>
       <c r="D14">
-        <v>7.786542131</v>
+        <v>7.7880382399999997</v>
       </c>
       <c r="E14">
-        <v>9.1743652999999897E-2</v>
+        <v>0.101517158</v>
       </c>
       <c r="F14">
-        <v>1.5035087389999899</v>
+        <v>1.512929634</v>
       </c>
       <c r="G14">
-        <v>5.8824202999999797E-2</v>
+        <v>5.6057263999999898E-2</v>
       </c>
       <c r="H14">
-        <v>8.0324217000000003E-2</v>
+        <v>0.458944827000001</v>
       </c>
       <c r="I14">
-        <v>0.14618890900000001</v>
+        <v>6.0638440610000002</v>
       </c>
       <c r="J14">
-        <v>0.22449387100000001</v>
+        <v>0.27262192800000001</v>
       </c>
       <c r="K14">
-        <v>0.145478408</v>
+        <v>0.491883189</v>
       </c>
       <c r="L14">
-        <v>1.510194391</v>
+        <v>3.895199383</v>
       </c>
       <c r="M14">
-        <v>1.9469330999999999E-2</v>
+        <v>1.947805E-2</v>
       </c>
       <c r="N14">
-        <v>0.55871432300000001</v>
+        <v>0.54294027499999997</v>
       </c>
       <c r="O14">
-        <v>11.602967883</v>
+        <v>20.697993238999999</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -3127,43 +3267,43 @@
         <v>21</v>
       </c>
       <c r="C15" s="1">
-        <v>2.0490970599999998E-2</v>
+        <v>2.1148022799999899E-2</v>
       </c>
       <c r="D15" s="1">
-        <v>7.7896655604999996</v>
+        <v>7.7888443829999998</v>
       </c>
       <c r="E15" s="1">
-        <v>9.1392076700000005E-2</v>
+        <v>0.1013372595</v>
       </c>
       <c r="F15" s="1">
-        <v>1.50496271489999</v>
+        <v>1.5131773657000001</v>
       </c>
       <c r="G15" s="1">
-        <v>5.7508319799999902E-2</v>
+        <v>5.5961258899999998E-2</v>
       </c>
       <c r="H15" s="1">
-        <v>8.0266894699999994E-2</v>
+        <v>0.45887892660000001</v>
       </c>
       <c r="I15" s="1">
-        <v>0.14648018700000001</v>
+        <v>6.0627548560999998</v>
       </c>
       <c r="J15" s="1">
-        <v>0.22424833150000001</v>
+        <v>0.27224948490000001</v>
       </c>
       <c r="K15" s="1">
-        <v>0.1457526992</v>
+        <v>0.49188873370000002</v>
       </c>
       <c r="L15" s="1">
-        <v>1.5127066299</v>
+        <v>3.8996550481000001</v>
       </c>
       <c r="M15" s="1">
-        <v>1.93910095E-2</v>
+        <v>1.9472640100000001E-2</v>
       </c>
       <c r="N15" s="1">
-        <v>0.57490099240000003</v>
+        <v>0.55042533940000005</v>
       </c>
       <c r="O15" s="1">
-        <v>11.6087681536</v>
+        <v>20.701861121499999</v>
       </c>
     </row>
   </sheetData>
@@ -3261,43 +3401,43 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>2.1670388999999901E-2</v>
+        <v>2.1042589E-2</v>
       </c>
       <c r="D5">
-        <v>7.788605767</v>
+        <v>7.7889424449999902</v>
       </c>
       <c r="E5">
-        <v>9.9566999999999795E-2</v>
+        <v>0.100951946999999</v>
       </c>
       <c r="F5">
-        <v>1.51476287599999</v>
+        <v>1.5158345339999999</v>
       </c>
       <c r="G5">
-        <v>5.6594470000000001E-2</v>
+        <v>5.5972837000000199E-2</v>
       </c>
       <c r="H5">
-        <v>0.45763494700000001</v>
+        <v>0.45902342800000101</v>
       </c>
       <c r="I5">
-        <v>6.0642653989999999</v>
+        <v>6.0615342429999997</v>
       </c>
       <c r="J5">
-        <v>0.27255439599999898</v>
+        <v>0.27380757500000003</v>
       </c>
       <c r="K5">
-        <v>0.49231615699999998</v>
+        <v>0.49236302999999798</v>
       </c>
       <c r="L5">
-        <v>3.9079429750000001</v>
+        <v>3.9015166990000001</v>
       </c>
       <c r="M5">
-        <v>2.0160246999999999E-2</v>
+        <v>1.9348687999999899E-2</v>
       </c>
       <c r="N5">
-        <v>0.62630026999999999</v>
+        <v>0.61524506599999995</v>
       </c>
       <c r="O5">
-        <v>20.713497519000001</v>
+        <v>20.706959798</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -3305,43 +3445,43 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>2.19130099999999E-2</v>
+        <v>2.1353419999999901E-2</v>
       </c>
       <c r="D6">
-        <v>7.79280851900001</v>
+        <v>7.79279711299999</v>
       </c>
       <c r="E6">
-        <v>9.9675741000000095E-2</v>
+        <v>0.101451716999999</v>
       </c>
       <c r="F6">
-        <v>1.514690286</v>
+        <v>1.5155008459999999</v>
       </c>
       <c r="G6">
-        <v>5.6976826000000001E-2</v>
+        <v>5.6154192000000103E-2</v>
       </c>
       <c r="H6">
-        <v>0.45819648799999901</v>
+        <v>0.45903085100000002</v>
       </c>
       <c r="I6">
-        <v>6.0626823300000003</v>
+        <v>6.0616481880000004</v>
       </c>
       <c r="J6">
-        <v>0.274515538</v>
+        <v>0.27378674200000003</v>
       </c>
       <c r="K6">
-        <v>0.49315212899999999</v>
+        <v>0.492847905999999</v>
       </c>
       <c r="L6">
-        <v>3.900064135</v>
+        <v>3.8941756330000001</v>
       </c>
       <c r="M6">
-        <v>2.0464525000000001E-2</v>
+        <v>1.9657917999999899E-2</v>
       </c>
       <c r="N6">
-        <v>0.54645062600000005</v>
+        <v>0.54726605800000006</v>
       </c>
       <c r="O6">
-        <v>20.712612427</v>
+        <v>20.704733495999999</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -3349,43 +3489,43 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>2.1715781E-2</v>
+        <v>2.0981407000000001E-2</v>
       </c>
       <c r="D7">
-        <v>7.78769075099998</v>
+        <v>7.7878332510000199</v>
       </c>
       <c r="E7">
-        <v>9.8289989999999897E-2</v>
+        <v>0.10093611299999999</v>
       </c>
       <c r="F7">
-        <v>1.51437557399999</v>
+        <v>1.515356916</v>
       </c>
       <c r="G7">
-        <v>5.6514841000000003E-2</v>
+        <v>5.5867665999999899E-2</v>
       </c>
       <c r="H7">
-        <v>0.45803918399999999</v>
+        <v>0.45886558199999899</v>
       </c>
       <c r="I7">
-        <v>6.0630073089999899</v>
+        <v>6.0629193100000096</v>
       </c>
       <c r="J7">
-        <v>0.27229793999999902</v>
+        <v>0.272240977</v>
       </c>
       <c r="K7">
-        <v>0.49229077099999902</v>
+        <v>0.49222443199999999</v>
       </c>
       <c r="L7">
-        <v>3.9083897669999899</v>
+        <v>3.8956862029999999</v>
       </c>
       <c r="M7">
-        <v>2.0096164E-2</v>
+        <v>1.9402821000000001E-2</v>
       </c>
       <c r="N7">
-        <v>0.54734508500000001</v>
+        <v>0.55455117300000001</v>
       </c>
       <c r="O7">
-        <v>20.709862891</v>
+        <v>20.698519548</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -3393,43 +3533,43 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>2.1558777000000001E-2</v>
+        <v>2.0956864999999901E-2</v>
       </c>
       <c r="D8">
-        <v>7.7885421700000004</v>
+        <v>7.7949866609999896</v>
       </c>
       <c r="E8">
-        <v>9.7385553000000097E-2</v>
+        <v>0.101300022</v>
       </c>
       <c r="F8">
-        <v>1.5140554819999901</v>
+        <v>1.51590531099999</v>
       </c>
       <c r="G8">
-        <v>5.6435298999999897E-2</v>
+        <v>5.5848188000000097E-2</v>
       </c>
       <c r="H8">
-        <v>0.45793884199999901</v>
+        <v>0.458857927</v>
       </c>
       <c r="I8">
-        <v>6.064377371</v>
+        <v>6.0650248729999898</v>
       </c>
       <c r="J8">
-        <v>0.27229752899999998</v>
+        <v>0.271976990999999</v>
       </c>
       <c r="K8">
-        <v>0.492120908999999</v>
+        <v>0.49213513599999997</v>
       </c>
       <c r="L8">
-        <v>3.9084012960000001</v>
+        <v>3.8964746520000002</v>
       </c>
       <c r="M8">
-        <v>1.9987675999999999E-2</v>
+        <v>1.9164344999999899E-2</v>
       </c>
       <c r="N8">
-        <v>0.55720628400000005</v>
+        <v>0.548205426</v>
       </c>
       <c r="O8">
-        <v>20.710153963</v>
+        <v>20.708969687</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -3437,43 +3577,43 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>2.1566398000000001E-2</v>
+        <v>2.0996747E-2</v>
       </c>
       <c r="D9">
-        <v>7.7886827629999997</v>
+        <v>7.7998079390000097</v>
       </c>
       <c r="E9">
-        <v>9.7693707000000005E-2</v>
+        <v>0.10090756400000001</v>
       </c>
       <c r="F9">
-        <v>1.5148509079999899</v>
+        <v>1.5161694799999901</v>
       </c>
       <c r="G9">
-        <v>5.6489028999999899E-2</v>
+        <v>5.5789725999999998E-2</v>
       </c>
       <c r="H9">
-        <v>0.45799976599999997</v>
+        <v>0.45893492999999902</v>
       </c>
       <c r="I9">
-        <v>6.0669434850000004</v>
+        <v>6.0662951339999998</v>
       </c>
       <c r="J9">
-        <v>0.27245112300000002</v>
+        <v>0.27210715099999999</v>
       </c>
       <c r="K9">
-        <v>0.49225550400000001</v>
+        <v>0.49207820800000002</v>
       </c>
       <c r="L9">
-        <v>3.9067603819999901</v>
+        <v>3.8898433239999899</v>
       </c>
       <c r="M9">
-        <v>2.00978629999999E-2</v>
+        <v>1.9294316999999998E-2</v>
       </c>
       <c r="N9">
-        <v>0.54859861300000001</v>
+        <v>0.55612084299999998</v>
       </c>
       <c r="O9">
-        <v>20.713437281000001</v>
+        <v>20.708475618000001</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -3481,43 +3621,43 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>2.1632118999999901E-2</v>
+        <v>2.0857225999999899E-2</v>
       </c>
       <c r="D10">
-        <v>7.7915927429999901</v>
+        <v>7.7925777399999898</v>
       </c>
       <c r="E10">
-        <v>9.7113913000000093E-2</v>
+        <v>0.100856243</v>
       </c>
       <c r="F10">
-        <v>1.51434344799999</v>
+        <v>1.5150176310000001</v>
       </c>
       <c r="G10">
-        <v>5.64154830000001E-2</v>
+        <v>5.5715932000000003E-2</v>
       </c>
       <c r="H10">
-        <v>0.45765355000000002</v>
+        <v>0.45881665199999999</v>
       </c>
       <c r="I10">
-        <v>6.0666592069999998</v>
+        <v>6.0656675150000003</v>
       </c>
       <c r="J10">
-        <v>0.271916721999999</v>
+        <v>0.271613084</v>
       </c>
       <c r="K10">
-        <v>0.493578724999999</v>
+        <v>0.492251412</v>
       </c>
       <c r="L10">
-        <v>3.90671174799999</v>
+        <v>3.9026557720000001</v>
       </c>
       <c r="M10">
-        <v>2.0044738999999999E-2</v>
+        <v>1.91470919999999E-2</v>
       </c>
       <c r="N10">
-        <v>0.54808315500000004</v>
+        <v>0.54054987300000001</v>
       </c>
       <c r="O10">
-        <v>20.715232767</v>
+        <v>20.71121874</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -3525,43 +3665,43 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>2.1658759999999899E-2</v>
+        <v>2.1145300999999901E-2</v>
       </c>
       <c r="D11">
-        <v>7.7947981879999997</v>
+        <v>7.7946861409999801</v>
       </c>
       <c r="E11">
-        <v>9.8980616000000105E-2</v>
+        <v>0.10150352999999999</v>
       </c>
       <c r="F11">
-        <v>1.5148128999999999</v>
+        <v>1.5156918319999999</v>
       </c>
       <c r="G11">
-        <v>5.6672052000000001E-2</v>
+        <v>5.5788429E-2</v>
       </c>
       <c r="H11">
-        <v>0.457924215999999</v>
+        <v>0.45897850600000001</v>
       </c>
       <c r="I11">
-        <v>6.0668586840000103</v>
+        <v>6.0672738399999897</v>
       </c>
       <c r="J11">
-        <v>0.272893575</v>
+        <v>0.27248283299999998</v>
       </c>
       <c r="K11">
-        <v>0.492327072999999</v>
+        <v>0.49234507700000002</v>
       </c>
       <c r="L11">
-        <v>3.9048722989999902</v>
+        <v>3.90366275199999</v>
       </c>
       <c r="M11">
-        <v>2.0216452999999999E-2</v>
+        <v>1.94385929999999E-2</v>
       </c>
       <c r="N11">
-        <v>0.54761473100000002</v>
+        <v>0.54143225800000006</v>
       </c>
       <c r="O11">
-        <v>20.719440948999999</v>
+        <v>20.719628178000001</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -3569,43 +3709,43 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>2.1639038999999999E-2</v>
+        <v>2.1019667999999998E-2</v>
       </c>
       <c r="D12">
-        <v>7.7899716459999997</v>
+        <v>7.7841760030000096</v>
       </c>
       <c r="E12">
-        <v>9.8083506999999903E-2</v>
+        <v>0.101018384</v>
       </c>
       <c r="F12">
-        <v>1.5127594169999901</v>
+        <v>1.5131399320000001</v>
       </c>
       <c r="G12">
-        <v>5.6608270000000002E-2</v>
+        <v>5.5908588000000099E-2</v>
       </c>
       <c r="H12">
-        <v>0.45777858199999899</v>
+        <v>0.45871410000000001</v>
       </c>
       <c r="I12">
-        <v>6.0622548540000096</v>
+        <v>6.0621998450000003</v>
       </c>
       <c r="J12">
-        <v>0.27232184799999998</v>
+        <v>0.27208021499999901</v>
       </c>
       <c r="K12">
-        <v>0.49182620599999899</v>
+        <v>0.491994816</v>
       </c>
       <c r="L12">
-        <v>3.9037054969999998</v>
+        <v>3.9061300939999999</v>
       </c>
       <c r="M12">
-        <v>2.0026265000000001E-2</v>
+        <v>1.9380764000000002E-2</v>
       </c>
       <c r="N12">
-        <v>0.54539367400000005</v>
+        <v>0.53954938200000002</v>
       </c>
       <c r="O12">
-        <v>20.704204261000001</v>
+        <v>20.702092305000001</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -3613,43 +3753,43 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>2.1713296999999999E-2</v>
+        <v>2.1795710999999902E-2</v>
       </c>
       <c r="D13">
-        <v>7.787347113</v>
+        <v>7.7842876979999804</v>
       </c>
       <c r="E13">
-        <v>9.7883269000000106E-2</v>
+        <v>0.100048781999999</v>
       </c>
       <c r="F13">
-        <v>1.51182173999999</v>
+        <v>1.5122951069999999</v>
       </c>
       <c r="G13">
-        <v>5.6496790999999998E-2</v>
+        <v>5.6704179000000098E-2</v>
       </c>
       <c r="H13">
-        <v>0.45767707799999902</v>
+        <v>0.45760545999999902</v>
       </c>
       <c r="I13">
-        <v>6.0607472580000001</v>
+        <v>6.060382626</v>
       </c>
       <c r="J13">
-        <v>0.27223769999999903</v>
+        <v>0.27251588799999898</v>
       </c>
       <c r="K13">
-        <v>0.49176235600000001</v>
+        <v>0.49164730800000001</v>
       </c>
       <c r="L13">
-        <v>3.89744741999999</v>
+        <v>3.9049001079999899</v>
       </c>
       <c r="M13">
-        <v>2.0108869000000001E-2</v>
+        <v>2.0220420999999999E-2</v>
       </c>
       <c r="N13">
-        <v>0.55015700700000003</v>
+        <v>0.56252935400000004</v>
       </c>
       <c r="O13">
-        <v>20.692585380000001</v>
+        <v>20.699717342</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -3657,43 +3797,43 @@
         <v>9</v>
       </c>
       <c r="C14">
-        <v>2.1855028999999901E-2</v>
+        <v>2.1231373000000001E-2</v>
       </c>
       <c r="D14">
-        <v>7.7860668789999696</v>
+        <v>7.7825284329999702</v>
       </c>
       <c r="E14">
-        <v>9.8922446999999997E-2</v>
+        <v>0.101947862</v>
       </c>
       <c r="F14">
-        <v>1.51220889299999</v>
+        <v>1.512921725</v>
       </c>
       <c r="G14">
-        <v>5.6745841999999901E-2</v>
+        <v>5.5964560999999899E-2</v>
       </c>
       <c r="H14">
-        <v>0.45806612199999902</v>
+        <v>0.45894390499999899</v>
       </c>
       <c r="I14">
-        <v>6.0625395729999996</v>
+        <v>6.0632913069999903</v>
       </c>
       <c r="J14">
-        <v>0.27311042299999999</v>
+        <v>0.27248361399999999</v>
       </c>
       <c r="K14">
-        <v>0.49177879899999999</v>
+        <v>0.49159298099999899</v>
       </c>
       <c r="L14">
-        <v>3.9069553799999999</v>
+        <v>3.9014519409999999</v>
       </c>
       <c r="M14">
-        <v>2.0284541999999999E-2</v>
+        <v>1.9455838E-2</v>
       </c>
       <c r="N14">
-        <v>0.54779951900000001</v>
+        <v>0.54230343400000003</v>
       </c>
       <c r="O14">
-        <v>20.705948580000001</v>
+        <v>20.698155360000001</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -3701,43 +3841,43 @@
         <v>21</v>
       </c>
       <c r="C15" s="1">
-        <v>2.16922599E-2</v>
+        <v>2.1138030700000001E-2</v>
       </c>
       <c r="D15" s="1">
-        <v>7.7896106538999899</v>
+        <v>7.7902623423999904</v>
       </c>
       <c r="E15" s="1">
-        <v>9.8359574300000002E-2</v>
+        <v>0.1010922164</v>
       </c>
       <c r="F15" s="1">
-        <v>1.51386815239999</v>
+        <v>1.5147833314000001</v>
       </c>
       <c r="G15" s="1">
-        <v>5.6594890299999999E-2</v>
+        <v>5.59714298E-2</v>
       </c>
       <c r="H15" s="1">
-        <v>0.45789087749999902</v>
+        <v>0.45877713409999998</v>
       </c>
       <c r="I15" s="1">
-        <v>6.0640335470000002</v>
+        <v>6.0636236880999999</v>
       </c>
       <c r="J15" s="1">
-        <v>0.27265967940000002</v>
+        <v>0.27250950699999998</v>
       </c>
       <c r="K15" s="1">
-        <v>0.49234086289999901</v>
+        <v>0.49214803059999901</v>
       </c>
       <c r="L15" s="1">
-        <v>3.9051250898999901</v>
+        <v>3.8996497178</v>
       </c>
       <c r="M15" s="1">
-        <v>2.0148734299999999E-2</v>
+        <v>1.9451079699999999E-2</v>
       </c>
       <c r="N15" s="1">
-        <v>0.55649489640000005</v>
+        <v>0.55477528669999998</v>
       </c>
       <c r="O15" s="1">
-        <v>20.709697601799999</v>
+        <v>20.705847007199999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add postprocessing and analysis of results
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F29E3D8-7825-7447-8785-B14548994AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914623F3-FD16-FA48-9026-C65353E34719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="56320" yWindow="0" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
+    <workbookView xWindow="1940" yWindow="1040" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_Results" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="61">
   <si>
     <t>Branch</t>
   </si>
@@ -121,6 +121,111 @@
   </si>
   <si>
     <t>Track reseeding</t>
+  </si>
+  <si>
+    <t>Atlas</t>
+  </si>
+  <si>
+    <t>run</t>
+  </si>
+  <si>
+    <t>along-step-neutral</t>
+  </si>
+  <si>
+    <t>along-step-uniform-msc</t>
+  </si>
+  <si>
+    <t>initialize-tracks</t>
+  </si>
+  <si>
+    <t>4.739928893000003</t>
+  </si>
+  <si>
+    <t>14.157920361000004</t>
+  </si>
+  <si>
+    <t>1.0943939320000016</t>
+  </si>
+  <si>
+    <t>4.8677925869999825</t>
+  </si>
+  <si>
+    <t>18.495831963000015</t>
+  </si>
+  <si>
+    <t>1.1414978990000058</t>
+  </si>
+  <si>
+    <t>4.539082406000011</t>
+  </si>
+  <si>
+    <t>14.07058440100002</t>
+  </si>
+  <si>
+    <t>1.0826401049999994</t>
+  </si>
+  <si>
+    <t>4.668021015000011</t>
+  </si>
+  <si>
+    <t>14.893830847000004</t>
+  </si>
+  <si>
+    <t>1.108715906000003</t>
+  </si>
+  <si>
+    <t>4.716793254999993</t>
+  </si>
+  <si>
+    <t>14.763301993999992</t>
+  </si>
+  <si>
+    <t>1.1058321380000014</t>
+  </si>
+  <si>
+    <t>4.854639256000009</t>
+  </si>
+  <si>
+    <t>14.163557716000016</t>
+  </si>
+  <si>
+    <t>1.0933890839999998</t>
+  </si>
+  <si>
+    <t>4.778291417000004</t>
+  </si>
+  <si>
+    <t>15.691015406000004</t>
+  </si>
+  <si>
+    <t>1.0883493359999996</t>
+  </si>
+  <si>
+    <t>4.617111119999994</t>
+  </si>
+  <si>
+    <t>15.159481652999983</t>
+  </si>
+  <si>
+    <t>1.088345942000003</t>
+  </si>
+  <si>
+    <t>4.672728067000012</t>
+  </si>
+  <si>
+    <t>15.186083537000004</t>
+  </si>
+  <si>
+    <t>1.122389057000007</t>
+  </si>
+  <si>
+    <t>4.704523719000007</t>
+  </si>
+  <si>
+    <t>13.082084631999992</t>
+  </si>
+  <si>
+    <t>1.1098299730000005</t>
   </si>
 </sst>
 </file>
@@ -169,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -179,6 +284,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B71848BA-D8C3-7041-A0EE-B663A4811CD2}">
-  <dimension ref="A1:AO19"/>
+  <dimension ref="A1:AO22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="42.1640625" bestFit="1" customWidth="1"/>
@@ -1148,27 +1255,298 @@
         <v>-2.3864001774150271E-2</v>
       </c>
     </row>
+    <row r="10" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="C10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+      <c r="X10" s="5"/>
+      <c r="Y10" s="5"/>
+      <c r="Z10" s="5"/>
+      <c r="AA10" s="5"/>
+      <c r="AB10" s="5"/>
+      <c r="AC10" s="5"/>
+      <c r="AD10" s="5"/>
+      <c r="AE10" s="5"/>
+      <c r="AF10" s="5"/>
+      <c r="AG10" s="5"/>
+      <c r="AH10" s="5"/>
+      <c r="AI10" s="5"/>
+      <c r="AJ10" s="5"/>
+      <c r="AK10" s="5"/>
+      <c r="AL10" s="5"/>
+      <c r="AM10" s="5"/>
+      <c r="AN10" s="5"/>
+      <c r="AO10" s="5"/>
+    </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="C11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B12" s="1"/>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L12" t="s">
+        <v>18</v>
+      </c>
+      <c r="M12" t="s">
+        <v>19</v>
+      </c>
+      <c r="N12" t="s">
+        <v>23</v>
+      </c>
+      <c r="O12" t="s">
+        <v>18</v>
+      </c>
+      <c r="P12" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="D13" s="1"/>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1">
+        <v>4.7158911735000002</v>
+      </c>
+      <c r="D13" s="1">
+        <v>4.6291748970000004</v>
+      </c>
+      <c r="E13">
+        <f>((C13-D13)/C13)*100</f>
+        <v>1.8388099578566284</v>
+      </c>
+      <c r="F13" s="1">
+        <v>14.966369251</v>
+      </c>
+      <c r="G13" s="1">
+        <v>15.464017373900001</v>
+      </c>
+      <c r="H13">
+        <f>((F13-G13)/F13)*100</f>
+        <v>-3.3251092135572562</v>
+      </c>
+      <c r="I13" s="1">
+        <v>1.1035383372000001</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1.1174958406</v>
+      </c>
+      <c r="K13">
+        <f>((I13-J13)/I13)*100</f>
+        <v>-1.264795515433943</v>
+      </c>
+      <c r="L13" s="1">
+        <v>45.087971282799998</v>
+      </c>
+      <c r="M13" s="1">
+        <v>44.8257993271</v>
+      </c>
+      <c r="N13">
+        <f>((L13-M13)/L13)*100</f>
+        <v>0.5814676248252717</v>
+      </c>
+      <c r="O13" s="1">
+        <v>21.769039145499999</v>
+      </c>
+      <c r="P13" s="1">
+        <v>22.5076772191</v>
+      </c>
+      <c r="Q13">
+        <f>((O13-P13)/O13)*100</f>
+        <v>-3.3930669546923422</v>
+      </c>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B14" s="1"/>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1">
+        <v>4.6941893570999902</v>
+      </c>
+      <c r="D14" s="1">
+        <v>4.6335907109000001</v>
+      </c>
+      <c r="E14">
+        <f>((C14-D14)/C14)*100</f>
+        <v>1.2909288822858049</v>
+      </c>
+      <c r="F14" s="1">
+        <v>14.3304367599</v>
+      </c>
+      <c r="G14" s="1">
+        <v>15.5303682837</v>
+      </c>
+      <c r="H14">
+        <f>((F14-G14)/F14)*100</f>
+        <v>-8.3733074148702595</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1.1054981386</v>
+      </c>
+      <c r="J14" s="1">
+        <v>1.1140971225</v>
+      </c>
+      <c r="K14">
+        <f>((I14-J14)/I14)*100</f>
+        <v>-0.77783793565584414</v>
+      </c>
+      <c r="L14" s="1">
+        <v>44.914485792800001</v>
+      </c>
+      <c r="M14" s="1">
+        <v>44.739087787199999</v>
+      </c>
+      <c r="N14">
+        <f>((L14-M14)/L14)*100</f>
+        <v>0.39051544842158442</v>
+      </c>
+      <c r="O14" s="1">
+        <v>21.1182229148</v>
+      </c>
+      <c r="P14" s="1">
+        <v>22.523737777600001</v>
+      </c>
+      <c r="Q14">
+        <f>((O14-P14)/O14)*100</f>
+        <v>-6.6554599242107271</v>
+      </c>
       <c r="T14" s="2"/>
     </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15">
+        <f>((C13-C14)/C13)*100</f>
+        <v>0.46018484315242458</v>
+      </c>
+      <c r="D15">
+        <f>((D13-D14)/D13)*100</f>
+        <v>-9.5390949753516641E-2</v>
+      </c>
+      <c r="F15">
+        <f>((F13-F14)/F13)*100</f>
+        <v>4.2490765825352694</v>
+      </c>
+      <c r="G15">
+        <f>((G13-G14)/G13)*100</f>
+        <v>-0.42906644629089163</v>
+      </c>
+      <c r="I15">
+        <f>((I13-I14)/I13)*100</f>
+        <v>-0.17759250711421146</v>
+      </c>
+      <c r="J15">
+        <f>((J13-J14)/J13)*100</f>
+        <v>0.30413697989024269</v>
+      </c>
+      <c r="L15">
+        <f>((L13-L14)/L13)*100</f>
+        <v>0.38477111536437214</v>
+      </c>
+      <c r="M15">
+        <f>((M13-M14)/M13)*100</f>
+        <v>0.19344114595091852</v>
+      </c>
+      <c r="O15">
+        <f>((O13-O14)/O13)*100</f>
+        <v>2.9896415103582208</v>
+      </c>
+      <c r="P15">
+        <f>((P13-P14)/P13)*100</f>
+        <v>-7.1355912667755608E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="D22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="20">
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="C10:Q10"/>
     <mergeCell ref="AM2:AO2"/>
     <mergeCell ref="C1:AO1"/>
     <mergeCell ref="U2:W2"/>
@@ -1184,8 +1562,18 @@
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:T2"/>
   </mergeCells>
+  <conditionalFormatting sqref="C6">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D6">
-    <cfRule type="colorScale" priority="60">
+    <cfRule type="colorScale" priority="75">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1195,7 +1583,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E4:E5">
-    <cfRule type="colorScale" priority="74">
+    <cfRule type="colorScale" priority="89">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F6">
+    <cfRule type="colorScale" priority="39">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6">
+    <cfRule type="colorScale" priority="38">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1205,7 +1613,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H5">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6">
     <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6">
+    <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1215,7 +1643,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:K5">
-    <cfRule type="colorScale" priority="36">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M6">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1225,7 +1673,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:N5">
-    <cfRule type="colorScale" priority="35">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O6">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P6">
+    <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1235,7 +1703,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q5">
-    <cfRule type="colorScale" priority="34">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R6">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S6">
+    <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1245,7 +1733,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T4:T5">
-    <cfRule type="colorScale" priority="33">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U6">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V6">
+    <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1255,7 +1763,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W4:W5">
-    <cfRule type="colorScale" priority="32">
+    <cfRule type="colorScale" priority="47">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X6">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y6">
+    <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1265,7 +1793,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z4:Z5">
-    <cfRule type="colorScale" priority="31">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB6">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1275,7 +1823,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC4:AC5">
-    <cfRule type="colorScale" priority="30">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD6">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE6">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1285,7 +1853,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF4:AF5">
-    <cfRule type="colorScale" priority="29">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG6">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AH6">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1295,7 +1883,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI4:AI5">
-    <cfRule type="colorScale" priority="28">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ6">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK6">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1305,7 +1913,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL4:AL5">
-    <cfRule type="colorScale" priority="27">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM6">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF3500"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN6">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1315,7 +1943,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO4:AO5">
-    <cfRule type="colorScale" priority="26">
+    <cfRule type="colorScale" priority="41">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1324,8 +1952,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="C15">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1334,8 +1962,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6">
-    <cfRule type="colorScale" priority="24">
+  <conditionalFormatting sqref="D15">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F15">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1344,8 +1982,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G6">
-    <cfRule type="colorScale" priority="23">
+  <conditionalFormatting sqref="G15">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I15">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1354,8 +2002,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6">
-    <cfRule type="colorScale" priority="22">
+  <conditionalFormatting sqref="J15">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L15">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1364,8 +2022,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6">
-    <cfRule type="colorScale" priority="21">
+  <conditionalFormatting sqref="M15">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O15">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1374,8 +2042,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="P15">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13:E14">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1384,8 +2062,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M6">
-    <cfRule type="colorScale" priority="19">
+  <conditionalFormatting sqref="H13:H14">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1394,8 +2072,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O6">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="K13:K14">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1404,8 +2082,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P6">
-    <cfRule type="colorScale" priority="17">
+  <conditionalFormatting sqref="N13:N14">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -1414,157 +2092,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R6">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S6">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U6">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V6">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X6">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y6">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA6">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB6">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD6">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE6">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AG6">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AH6">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ6">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK6">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM6">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FFFF3500"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN6">
+  <conditionalFormatting sqref="Q13:Q14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1580,13 +2108,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D90E2C0-8C68-E84F-BBAA-6A32D2F1D90D}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.1640625" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
@@ -2158,9 +2686,281 @@
         <v>20.700766578500001</v>
       </c>
     </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20">
+        <v>45.178059114</v>
+      </c>
+      <c r="G20">
+        <v>20.935805562999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21">
+        <v>44.446670339999997</v>
+      </c>
+      <c r="G21">
+        <v>25.681944958999999</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22">
+        <v>44.993960194000003</v>
+      </c>
+      <c r="G22">
+        <v>20.587326808</v>
+      </c>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23">
+        <v>44.808145336999999</v>
+      </c>
+      <c r="G23">
+        <v>21.655821433</v>
+      </c>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24">
+        <v>44.748611527000001</v>
+      </c>
+      <c r="G24">
+        <v>21.545505545000001</v>
+      </c>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+    </row>
+    <row r="25" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25">
+        <v>44.639488767000003</v>
+      </c>
+      <c r="G25">
+        <v>21.058005052999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F26">
+        <v>44.722949407000002</v>
+      </c>
+      <c r="G26">
+        <v>22.522632615999999</v>
+      </c>
+    </row>
+    <row r="27" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27">
+        <v>44.645210781000003</v>
+      </c>
+      <c r="G27">
+        <v>21.857823479</v>
+      </c>
+    </row>
+    <row r="28" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>8</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F28">
+        <v>47.971052186999998</v>
+      </c>
+      <c r="G28">
+        <v>22.030840081000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>9</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29">
+        <v>44.725565174000003</v>
+      </c>
+      <c r="G29">
+        <v>19.814685917999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="1">
+        <v>4.7158911735000002</v>
+      </c>
+      <c r="D30" s="1">
+        <v>14.966369251</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1.1035383372000001</v>
+      </c>
+      <c r="F30" s="1">
+        <v>45.087971282799998</v>
+      </c>
+      <c r="G30" s="1">
+        <v>21.769039145499999</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C3:O3"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2168,8 +2968,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B17374F-425A-0C4A-B316-973C7C980C22}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -2732,9 +3539,260 @@
         <v>20.7009069424</v>
       </c>
     </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>4.8237869980000001</v>
+      </c>
+      <c r="D20">
+        <v>16.405531232999898</v>
+      </c>
+      <c r="E20">
+        <v>1.153891198</v>
+      </c>
+      <c r="F20">
+        <v>44.99530566</v>
+      </c>
+      <c r="G20">
+        <v>23.770921220999998</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>4.6673217520000003</v>
+      </c>
+      <c r="D21">
+        <v>14.449837002999899</v>
+      </c>
+      <c r="E21">
+        <v>1.1181004369999901</v>
+      </c>
+      <c r="F21">
+        <v>45.118839434999998</v>
+      </c>
+      <c r="G21">
+        <v>21.509625474</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>4.7014450299999897</v>
+      </c>
+      <c r="D22">
+        <v>15.184039253</v>
+      </c>
+      <c r="E22">
+        <v>1.1095911629999999</v>
+      </c>
+      <c r="F22">
+        <v>44.721127103000001</v>
+      </c>
+      <c r="G22">
+        <v>22.276340040000001</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>4.4885547370000003</v>
+      </c>
+      <c r="D23">
+        <v>15.4021777489999</v>
+      </c>
+      <c r="E23">
+        <v>1.10351937899999</v>
+      </c>
+      <c r="F23">
+        <v>44.616166184999997</v>
+      </c>
+      <c r="G23">
+        <v>22.257800827000001</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24">
+        <v>4.7220404680000003</v>
+      </c>
+      <c r="D24">
+        <v>16.394596872000001</v>
+      </c>
+      <c r="E24">
+        <v>1.12422092099999</v>
+      </c>
+      <c r="F24">
+        <v>44.595392926000002</v>
+      </c>
+      <c r="G24">
+        <v>23.554986079999999</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>4.8406276199999896</v>
+      </c>
+      <c r="D25">
+        <v>15.607468506999901</v>
+      </c>
+      <c r="E25">
+        <v>1.1448489749999899</v>
+      </c>
+      <c r="F25">
+        <v>44.5322107</v>
+      </c>
+      <c r="G25">
+        <v>22.953275693999998</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>4.4273572260000096</v>
+      </c>
+      <c r="D26">
+        <v>14.531455789000001</v>
+      </c>
+      <c r="E26">
+        <v>1.09781243699999</v>
+      </c>
+      <c r="F26">
+        <v>44.845106297000001</v>
+      </c>
+      <c r="G26">
+        <v>21.291217564</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27">
+        <v>4.4705501949999897</v>
+      </c>
+      <c r="D27">
+        <v>15.201100657</v>
+      </c>
+      <c r="E27">
+        <v>1.0945569470000001</v>
+      </c>
+      <c r="F27">
+        <v>44.662393252999998</v>
+      </c>
+      <c r="G27">
+        <v>21.995210685</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <v>4.59382215000001</v>
+      </c>
+      <c r="D28">
+        <v>15.862654592999901</v>
+      </c>
+      <c r="E28">
+        <v>1.1204468359999999</v>
+      </c>
+      <c r="F28">
+        <v>45.072985840999998</v>
+      </c>
+      <c r="G28">
+        <v>22.860605258</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>9</v>
+      </c>
+      <c r="C29">
+        <v>4.5562427940000001</v>
+      </c>
+      <c r="D29">
+        <v>15.6013120829999</v>
+      </c>
+      <c r="E29">
+        <v>1.1079701129999999</v>
+      </c>
+      <c r="F29">
+        <v>45.098465871000002</v>
+      </c>
+      <c r="G29">
+        <v>22.606789348</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="1">
+        <v>4.6291748970000004</v>
+      </c>
+      <c r="D30" s="1">
+        <v>15.464017373900001</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1.1174958406</v>
+      </c>
+      <c r="F30" s="1">
+        <v>44.8257993271</v>
+      </c>
+      <c r="G30" s="1">
+        <v>22.5076772191</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C3:O3"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2742,7 +3800,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE3BDD0-3A87-544A-A16E-D142A4C1F8FB}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -3306,9 +4364,267 @@
         <v>20.701861121499999</v>
       </c>
     </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>4.6006060579999897</v>
+      </c>
+      <c r="D20">
+        <v>15.542913898</v>
+      </c>
+      <c r="E20">
+        <v>1.0821381290000001</v>
+      </c>
+      <c r="F20">
+        <v>44.868074825000001</v>
+      </c>
+      <c r="G20">
+        <v>22.239466582999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>4.6237777609999897</v>
+      </c>
+      <c r="D21">
+        <v>14.005688256999999</v>
+      </c>
+      <c r="E21">
+        <v>1.0931326799999901</v>
+      </c>
+      <c r="F21">
+        <v>45.367524641000003</v>
+      </c>
+      <c r="G21">
+        <v>20.678480005000001</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>4.5162472820000001</v>
+      </c>
+      <c r="D22">
+        <v>14.3467801379999</v>
+      </c>
+      <c r="E22">
+        <v>1.1148718719999899</v>
+      </c>
+      <c r="F22">
+        <v>44.413765368</v>
+      </c>
+      <c r="G22">
+        <v>20.931622545</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>4.8416728419999897</v>
+      </c>
+      <c r="D23">
+        <v>14.1692157299999</v>
+      </c>
+      <c r="E23">
+        <v>1.12419611599999</v>
+      </c>
+      <c r="F23">
+        <v>45.201858715999997</v>
+      </c>
+      <c r="G23">
+        <v>21.150967145999999</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24">
+        <v>4.8448703529999904</v>
+      </c>
+      <c r="D24">
+        <v>13.885040346</v>
+      </c>
+      <c r="E24">
+        <v>1.1458932610000001</v>
+      </c>
+      <c r="F24">
+        <v>44.601139498000002</v>
+      </c>
+      <c r="G24">
+        <v>20.890493974999998</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>4.7523815999999899</v>
+      </c>
+      <c r="D25">
+        <v>14.416007534999901</v>
+      </c>
+      <c r="E25">
+        <v>1.104802775</v>
+      </c>
+      <c r="F25">
+        <v>44.893572736000003</v>
+      </c>
+      <c r="G25">
+        <v>21.308788703000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>4.7771238329999903</v>
+      </c>
+      <c r="D26">
+        <v>14.535514169000001</v>
+      </c>
+      <c r="E26">
+        <v>1.13063033</v>
+      </c>
+      <c r="F26">
+        <v>45.022300168999998</v>
+      </c>
+      <c r="G26">
+        <v>21.462349112999998</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27">
+        <v>4.6711723949999797</v>
+      </c>
+      <c r="D27">
+        <v>14.424652171999901</v>
+      </c>
+      <c r="E27">
+        <v>1.07934710399999</v>
+      </c>
+      <c r="F27">
+        <v>45.100189931999999</v>
+      </c>
+      <c r="G27">
+        <v>21.122489199</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <v>4.5969812780000003</v>
+      </c>
+      <c r="D28">
+        <v>14.396043703999901</v>
+      </c>
+      <c r="E28">
+        <v>1.09079157099999</v>
+      </c>
+      <c r="F28">
+        <v>44.191400801</v>
+      </c>
+      <c r="G28">
+        <v>21.039077846000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>9</v>
+      </c>
+      <c r="C29">
+        <v>4.7170601689999998</v>
+      </c>
+      <c r="D29">
+        <v>13.582511649999899</v>
+      </c>
+      <c r="E29">
+        <v>1.0891775480000001</v>
+      </c>
+      <c r="F29">
+        <v>45.485031241999998</v>
+      </c>
+      <c r="G29">
+        <v>20.358494032999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="1">
+        <v>4.6941893570999902</v>
+      </c>
+      <c r="D30" s="1">
+        <v>14.3304367599</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1.1054981386</v>
+      </c>
+      <c r="F30" s="1">
+        <v>44.914485792800001</v>
+      </c>
+      <c r="G30" s="1">
+        <v>21.1182229148</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C3:O3"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3316,7 +4632,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBF611A7-FF5C-9946-82AC-26D645B98B8C}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -3880,9 +5196,260 @@
         <v>20.705847007199999</v>
       </c>
     </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>4.6821826419999999</v>
+      </c>
+      <c r="D20">
+        <v>15.9062169909999</v>
+      </c>
+      <c r="E20">
+        <v>1.121482047</v>
+      </c>
+      <c r="F20">
+        <v>44.397116122</v>
+      </c>
+      <c r="G20">
+        <v>22.945172749000001</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>4.9315779149999903</v>
+      </c>
+      <c r="D21">
+        <v>16.390990083999998</v>
+      </c>
+      <c r="E21">
+        <v>1.192110045</v>
+      </c>
+      <c r="F21">
+        <v>45.113467712999999</v>
+      </c>
+      <c r="G21">
+        <v>23.885588552000002</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>4.4953373430000001</v>
+      </c>
+      <c r="D22">
+        <v>15.650422679999901</v>
+      </c>
+      <c r="E22">
+        <v>1.1235293309999901</v>
+      </c>
+      <c r="F22">
+        <v>44.746627072000003</v>
+      </c>
+      <c r="G22">
+        <v>22.479247667999999</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>4.5581672070000003</v>
+      </c>
+      <c r="D23">
+        <v>14.377298114</v>
+      </c>
+      <c r="E23">
+        <v>1.10439433899999</v>
+      </c>
+      <c r="F23">
+        <v>45.184373686000001</v>
+      </c>
+      <c r="G23">
+        <v>21.237795102</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24">
+        <v>4.5335301469999996</v>
+      </c>
+      <c r="D24">
+        <v>15.151445159</v>
+      </c>
+      <c r="E24">
+        <v>1.0928487359999901</v>
+      </c>
+      <c r="F24">
+        <v>44.322336700000001</v>
+      </c>
+      <c r="G24">
+        <v>21.952346764000001</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>4.7823800330000097</v>
+      </c>
+      <c r="D25">
+        <v>15.646650354999901</v>
+      </c>
+      <c r="E25">
+        <v>1.1116416419999999</v>
+      </c>
+      <c r="F25">
+        <v>44.701800239000001</v>
+      </c>
+      <c r="G25">
+        <v>22.869030379000002</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>4.4649637659999897</v>
+      </c>
+      <c r="D26">
+        <v>15.741240229999899</v>
+      </c>
+      <c r="E26">
+        <v>1.0914018059999899</v>
+      </c>
+      <c r="F26">
+        <v>44.399810017</v>
+      </c>
+      <c r="G26">
+        <v>22.544032024</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27">
+        <v>4.7631122550000002</v>
+      </c>
+      <c r="D27">
+        <v>15.3062458429999</v>
+      </c>
+      <c r="E27">
+        <v>1.126965164</v>
+      </c>
+      <c r="F27">
+        <v>44.695782704000003</v>
+      </c>
+      <c r="G27">
+        <v>22.480037155000002</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <v>4.5826042339999997</v>
+      </c>
+      <c r="D28">
+        <v>15.840817636999899</v>
+      </c>
+      <c r="E28">
+        <v>1.099819111</v>
+      </c>
+      <c r="F28">
+        <v>45.131765295999998</v>
+      </c>
+      <c r="G28">
+        <v>22.729038668000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>9</v>
+      </c>
+      <c r="C29">
+        <v>4.5420515669999997</v>
+      </c>
+      <c r="D29">
+        <v>15.2923557439999</v>
+      </c>
+      <c r="E29">
+        <v>1.076779004</v>
+      </c>
+      <c r="F29">
+        <v>44.697798323000001</v>
+      </c>
+      <c r="G29">
+        <v>22.115088714999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="1">
+        <v>4.6335907109000001</v>
+      </c>
+      <c r="D30" s="1">
+        <v>15.5303682837</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1.1140971225</v>
+      </c>
+      <c r="F30" s="1">
+        <v>44.739087787199999</v>
+      </c>
+      <c r="G30" s="1">
+        <v>22.523737777600001</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C3:O3"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Working on Analysis notebook
</commit_message>
<xml_diff>
--- a/Analysis.xlsx
+++ b/Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gqe/Codes/celeritas/analysis/celer_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A87567-1EA1-4546-BBAC-E465585AE33D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AED7FF-68B8-274E-AA2B-435BFEA4FCC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="54880" yWindow="1100" windowWidth="47520" windowHeight="26040" xr2:uid="{18F4029D-343F-3648-AF31-0004853598C3}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="58">
   <si>
     <t>Branch</t>
   </si>
@@ -285,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -293,9 +293,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1292,47 +1289,59 @@
       </c>
       <c r="AO6" s="3"/>
     </row>
+    <row r="8" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="B8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B9" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
+      <c r="F10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="4">
+        <v>104</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
       <c r="T10" s="1"/>
       <c r="AB10" s="1"/>
       <c r="AC10" s="1"/>
@@ -1351,172 +1360,183 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="C11">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="D11">
+        <v>0.5</v>
+      </c>
+      <c r="E11">
+        <v>152</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="4">
+        <v>128</v>
+      </c>
+      <c r="H11" s="4">
         <v>0.25</v>
       </c>
-      <c r="E11">
-        <v>0</v>
+      <c r="I11" s="4">
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12">
-        <v>128</v>
+        <v>47</v>
       </c>
       <c r="D12">
-        <v>0.25</v>
+        <v>0.625</v>
       </c>
       <c r="E12">
-        <v>144</v>
-      </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="4">
         <v>64</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="4">
         <v>0.5</v>
       </c>
-      <c r="I12">
-        <v>152</v>
+      <c r="I12" s="4">
+        <v>8</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="C13">
+        <v>48</v>
+      </c>
+      <c r="D13">
+        <v>0.625</v>
+      </c>
+      <c r="E13">
         <v>64</v>
       </c>
-      <c r="D13">
-        <v>0.5</v>
-      </c>
-      <c r="E13">
-        <v>8</v>
-      </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13">
-        <v>47</v>
-      </c>
-      <c r="H13">
-        <v>0.625</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
+      <c r="F13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="4">
+        <v>110</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="I13" s="4">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14">
-        <v>110</v>
-      </c>
-      <c r="D14">
-        <v>0.25</v>
-      </c>
-      <c r="E14">
-        <v>64</v>
-      </c>
-      <c r="F14" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14">
-        <v>48</v>
-      </c>
-      <c r="H14">
-        <v>0.625</v>
-      </c>
-      <c r="I14">
-        <v>64</v>
-      </c>
+      <c r="B14" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
       <c r="T14" s="2"/>
       <c r="AB14" s="1"/>
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B15" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
+      <c r="B15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="B16" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="G16">
+        <v>104</v>
+      </c>
+      <c r="H16">
+        <v>0.25</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:59" x14ac:dyDescent="0.2">
-      <c r="B17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="4">
-        <v>104</v>
-      </c>
-      <c r="D17" s="4">
+      <c r="B17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>64</v>
+      </c>
+      <c r="D17">
+        <v>0.5</v>
+      </c>
+      <c r="E17">
+        <v>152</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17">
+        <v>128</v>
+      </c>
+      <c r="H17">
         <v>0.25</v>
       </c>
-      <c r="E17" s="4">
+      <c r="I17">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="2:59" x14ac:dyDescent="0.2">
+      <c r="B18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18">
+        <v>47</v>
+      </c>
+      <c r="D18">
+        <v>0.625</v>
+      </c>
+      <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="2:59" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="4">
-        <v>128</v>
-      </c>
-      <c r="D18" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="E18" s="4">
-        <v>144</v>
-      </c>
       <c r="F18" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G18">
         <v>64</v>
@@ -1525,58 +1545,32 @@
         <v>0.5</v>
       </c>
       <c r="I18">
-        <v>152</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="2:59" x14ac:dyDescent="0.2">
-      <c r="B19" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="4">
+      <c r="B19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19">
+        <v>48</v>
+      </c>
+      <c r="D19">
+        <v>0.625</v>
+      </c>
+      <c r="E19">
         <v>64</v>
       </c>
-      <c r="D19" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E19" s="4">
-        <v>8</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="G19">
-        <v>47</v>
+        <v>110</v>
       </c>
       <c r="H19">
-        <v>0.625</v>
+        <v>0.25</v>
       </c>
       <c r="I19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:59" x14ac:dyDescent="0.2">
-      <c r="B20" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="4">
-        <v>110</v>
-      </c>
-      <c r="D20" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="E20" s="4">
-        <v>64</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G20">
-        <v>48</v>
-      </c>
-      <c r="H20">
-        <v>0.625</v>
-      </c>
-      <c r="I20">
         <v>64</v>
       </c>
     </row>
@@ -2436,12 +2430,64 @@
       </c>
       <c r="BG27" s="3"/>
     </row>
+    <row r="30" spans="2:59" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="2:59" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31">
+        <v>80</v>
+      </c>
+      <c r="D31">
+        <v>0.375</v>
+      </c>
+      <c r="E31">
+        <v>32</v>
+      </c>
+    </row>
     <row r="35" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="AG23:AI23"/>
+    <mergeCell ref="AJ23:AL23"/>
+    <mergeCell ref="AM23:AO23"/>
+    <mergeCell ref="BE23:BG23"/>
+    <mergeCell ref="AP23:AR23"/>
+    <mergeCell ref="AS23:AU23"/>
+    <mergeCell ref="AV23:AX23"/>
+    <mergeCell ref="AY23:BA23"/>
+    <mergeCell ref="BB23:BD23"/>
+    <mergeCell ref="R23:T23"/>
+    <mergeCell ref="X23:Z23"/>
+    <mergeCell ref="U23:W23"/>
+    <mergeCell ref="AA23:AC23"/>
+    <mergeCell ref="AD23:AF23"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C22:Q22"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="AM2:AO2"/>
     <mergeCell ref="C1:AO1"/>
     <mergeCell ref="U2:W2"/>
@@ -2456,33 +2502,9 @@
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="R2:T2"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C22:Q22"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="L23:N23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="R23:T23"/>
-    <mergeCell ref="X23:Z23"/>
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="AA23:AC23"/>
-    <mergeCell ref="AD23:AF23"/>
-    <mergeCell ref="AG23:AI23"/>
-    <mergeCell ref="AJ23:AL23"/>
-    <mergeCell ref="AM23:AO23"/>
-    <mergeCell ref="BE23:BG23"/>
-    <mergeCell ref="AP23:AR23"/>
-    <mergeCell ref="AS23:AU23"/>
-    <mergeCell ref="AV23:AX23"/>
-    <mergeCell ref="AY23:BA23"/>
-    <mergeCell ref="BB23:BD23"/>
   </mergeCells>
-  <conditionalFormatting sqref="C27:D27">
-    <cfRule type="colorScale" priority="135">
+  <conditionalFormatting sqref="C6:D6">
+    <cfRule type="colorScale" priority="161">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2491,8 +2513,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:D6">
-    <cfRule type="colorScale" priority="161">
+  <conditionalFormatting sqref="C27:D27">
+    <cfRule type="colorScale" priority="135">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2521,8 +2543,58 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F6:G6">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F27:G27">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H4:H5">
     <cfRule type="colorScale" priority="60">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25:H26">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:J6">
+    <cfRule type="colorScale" priority="47">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I27:J27">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2541,8 +2613,68 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K25:K26">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6:M6">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L27:M27">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="N4:N5">
     <cfRule type="colorScale" priority="58">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N25:N26">
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O6:P6">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O27:P27">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2561,8 +2693,68 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q25:Q26">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R6:S6">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R27:S27">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="T4:T5">
     <cfRule type="colorScale" priority="56">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T25:T26">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U6:V6">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U27:V27">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2581,8 +2773,68 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W25:W26">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X6:Y6">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X27:Y27">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="Z4:Z5">
     <cfRule type="colorScale" priority="54">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z25:Z26">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6:AB6">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA27:AB27">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2601,8 +2853,68 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AC25:AC26">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD6:AE6">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD27:AE27">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AF4:AF5">
     <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF25:AF26">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG6:AH6">
+    <cfRule type="colorScale" priority="39">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG27:AH27">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2621,8 +2933,68 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AI25:AI26">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ6:AK6">
+    <cfRule type="colorScale" priority="38">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ27:AK27">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AL4:AL5">
     <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL25:AL26">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM6:AN6">
+    <cfRule type="colorScale" priority="37">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM27:AN27">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2641,8 +3013,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F6:G6">
-    <cfRule type="colorScale" priority="48">
+  <conditionalFormatting sqref="AO25:AO26">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2651,228 +3023,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J6">
-    <cfRule type="colorScale" priority="47">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L6:M6">
-    <cfRule type="colorScale" priority="46">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O6:P6">
-    <cfRule type="colorScale" priority="45">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R6:S6">
-    <cfRule type="colorScale" priority="44">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U6:V6">
-    <cfRule type="colorScale" priority="43">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X6:Y6">
-    <cfRule type="colorScale" priority="42">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA6:AB6">
-    <cfRule type="colorScale" priority="41">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD6:AE6">
-    <cfRule type="colorScale" priority="40">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AG6:AH6">
-    <cfRule type="colorScale" priority="39">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ6:AK6">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM6:AN6">
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H25:H26">
-    <cfRule type="colorScale" priority="36">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K25:K26">
-    <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N25:N26">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q25:Q26">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T25:T26">
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W25:W26">
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z25:Z26">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC25:AC26">
-    <cfRule type="colorScale" priority="29">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AF25:AF26">
-    <cfRule type="colorScale" priority="28">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI25:AI26">
-    <cfRule type="colorScale" priority="27">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL25:AL26">
-    <cfRule type="colorScale" priority="26">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO25:AO26">
-    <cfRule type="colorScale" priority="25">
+  <conditionalFormatting sqref="AP27:AQ27">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2891,8 +3043,28 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AS27:AT27">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AU25:AU26">
     <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AV27:AW27">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2911,8 +3083,28 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AY27:AZ27">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="BA25:BA26">
     <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color rgb="FF92D050"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BB27:BC27">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2931,8 +3123,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BG25:BG26">
-    <cfRule type="colorScale" priority="19">
+  <conditionalFormatting sqref="BE27:BF27">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2941,178 +3133,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27:G27">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I27:J27">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L27:M27">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O27:P27">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R27:S27">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U27:V27">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X27:Y27">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA27:AB27">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD27:AE27">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AG27:AH27">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ27:AK27">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM27:AN27">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP27:AQ27">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AS27:AT27">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AV27:AW27">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AY27:AZ27">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BB27:BC27">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color rgb="FF92D050"/>
-        <color rgb="FFFF0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="BE27:BF27">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="BG25:BG26">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>

</xml_diff>